<commit_message>
fix(template): v4 — recalc-on-load, 30-staff capacity, lead-gen contact line
- fullCalcOnLoad: formulas ship without cached values, so Protected View (every
  internet download) showed blank names/dates/outputs until Enable Editing +
  recalc; now everything populates the moment editing is enabled, and the
  Instructions explain the Protected View banner.
- Staff capacity 20 -> 30 unlocked roster rows; Schedule grid mirrors all 30
  with guarded formulas (unused rows stay blank, no zeros or false flags).
  Staff tab note: need more than 30 -> hello@simplescheduleai.com (founder's
  lead-gen line for the capacity ceiling).
- Week-start column widened (was rendering ####).
- Download link version bumped (?v=20260721b) to bypass the 4h edge cache.
- 41/41 formula tests + protection audit green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/SimpleScheduleAI-Nurse-Schedule-Template.xlsx
+++ b/public/downloads/SimpleScheduleAI-Nurse-Schedule-Template.xlsx
@@ -26,7 +26,7 @@
     <definedName name="DayCodes">Shifts!$A$2:$A$5</definedName>
     <definedName name="NightCodes">Shifts!$A$6:$A$8</definedName>
     <definedName name="OffCodes">Shifts!$A$9:$A$12</definedName>
-    <definedName name="StaffTbl">Staff!$A$2:$B$21</definedName>
+    <definedName name="StaffTbl">Staff!$A$2:$B$31</definedName>
     <definedName name="OT_Threshold">Rules!$B$2</definedName>
     <definedName name="Rest_Hours">Rules!$B$3</definedName>
     <definedName name="Max_Consecutive">Rules!$B$4</definedName>
@@ -80,6 +80,11 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="002D5A4A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00B00000"/>
     </font>
     <font>
@@ -94,11 +99,6 @@
     <font>
       <b val="1"/>
       <color rgb="002D5A4A"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="002D5A4A"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="5">
@@ -170,7 +170,7 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
@@ -179,11 +179,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -198,9 +201,6 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -220,12 +220,12 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -843,16 +843,16 @@
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    5.  Check the overtime flags and the coverage gap rows. Adjust until gaps are zero and no one is over threshold.</t>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>First open: Excel shows downloaded files in Protected View, where formulas display as blank cells. Click Enable Editing at the top and everything (names, dates, checks) fills in.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Notes: names on the Leave tab must match the Staff tab exactly. Consecutive-days and rest checks look at the displayed week only; they cannot see last week's shifts.</t>
+          <t>Notes: names on the Leave tab must match the Staff tab exactly. The roster holds up to 30 staff; add them on the Staff tab and they appear on the Schedule automatically. Need more than 30, or a version adapted to your hospital? Write to hello@simplescheduleai.com. Consecutive-days and rest checks look at the displayed week only; they cannot see last week's shifts.</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1706,6 +1706,130 @@
       </c>
       <c r="I21" s="9" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="n"/>
+      <c r="B22" s="10" t="n"/>
+      <c r="C22" s="10" t="n"/>
+      <c r="D22" s="10" t="n"/>
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="10" t="n"/>
+      <c r="G22" s="10" t="n"/>
+      <c r="H22" s="10" t="n"/>
+      <c r="I22" s="10" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="n"/>
+      <c r="B23" s="10" t="n"/>
+      <c r="C23" s="10" t="n"/>
+      <c r="D23" s="10" t="n"/>
+      <c r="E23" s="10" t="n"/>
+      <c r="F23" s="10" t="n"/>
+      <c r="G23" s="10" t="n"/>
+      <c r="H23" s="10" t="n"/>
+      <c r="I23" s="10" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="n"/>
+      <c r="B24" s="10" t="n"/>
+      <c r="C24" s="10" t="n"/>
+      <c r="D24" s="10" t="n"/>
+      <c r="E24" s="10" t="n"/>
+      <c r="F24" s="10" t="n"/>
+      <c r="G24" s="10" t="n"/>
+      <c r="H24" s="10" t="n"/>
+      <c r="I24" s="10" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="n"/>
+      <c r="B25" s="10" t="n"/>
+      <c r="C25" s="10" t="n"/>
+      <c r="D25" s="10" t="n"/>
+      <c r="E25" s="10" t="n"/>
+      <c r="F25" s="10" t="n"/>
+      <c r="G25" s="10" t="n"/>
+      <c r="H25" s="10" t="n"/>
+      <c r="I25" s="10" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="n"/>
+      <c r="B26" s="10" t="n"/>
+      <c r="C26" s="10" t="n"/>
+      <c r="D26" s="10" t="n"/>
+      <c r="E26" s="10" t="n"/>
+      <c r="F26" s="10" t="n"/>
+      <c r="G26" s="10" t="n"/>
+      <c r="H26" s="10" t="n"/>
+      <c r="I26" s="10" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="n"/>
+      <c r="B27" s="10" t="n"/>
+      <c r="C27" s="10" t="n"/>
+      <c r="D27" s="10" t="n"/>
+      <c r="E27" s="10" t="n"/>
+      <c r="F27" s="10" t="n"/>
+      <c r="G27" s="10" t="n"/>
+      <c r="H27" s="10" t="n"/>
+      <c r="I27" s="10" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="n"/>
+      <c r="B28" s="10" t="n"/>
+      <c r="C28" s="10" t="n"/>
+      <c r="D28" s="10" t="n"/>
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="10" t="n"/>
+      <c r="G28" s="10" t="n"/>
+      <c r="H28" s="10" t="n"/>
+      <c r="I28" s="10" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="n"/>
+      <c r="B29" s="10" t="n"/>
+      <c r="C29" s="10" t="n"/>
+      <c r="D29" s="10" t="n"/>
+      <c r="E29" s="10" t="n"/>
+      <c r="F29" s="10" t="n"/>
+      <c r="G29" s="10" t="n"/>
+      <c r="H29" s="10" t="n"/>
+      <c r="I29" s="10" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="n"/>
+      <c r="B30" s="10" t="n"/>
+      <c r="C30" s="10" t="n"/>
+      <c r="D30" s="10" t="n"/>
+      <c r="E30" s="10" t="n"/>
+      <c r="F30" s="10" t="n"/>
+      <c r="G30" s="10" t="n"/>
+      <c r="H30" s="10" t="n"/>
+      <c r="I30" s="10" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="n"/>
+      <c r="B31" s="10" t="n"/>
+      <c r="C31" s="10" t="n"/>
+      <c r="D31" s="10" t="n"/>
+      <c r="E31" s="10" t="n"/>
+      <c r="F31" s="10" t="n"/>
+      <c r="G31" s="10" t="n"/>
+      <c r="H31" s="10" t="n"/>
+      <c r="I31" s="10" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>Add more staff in the empty rows above (up to 30 total); they appear on the Schedule tab automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Need more than 30 staff, or a version adapted to your hospital? Write to us at hello@simplescheduleai.com and we will set you up.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1769,16 +1893,16 @@
           <t>Med-Surg</t>
         </is>
       </c>
-      <c r="B2" s="10" t="n">
+      <c r="B2" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="C2" s="10" t="n">
+      <c r="C2" s="12" t="n">
         <v>0.6</v>
       </c>
-      <c r="D2" s="10" t="n">
+      <c r="D2" s="12" t="n">
         <v>0.65</v>
       </c>
-      <c r="E2" s="10" t="n">
+      <c r="E2" s="12" t="n">
         <v>0.6</v>
       </c>
     </row>
@@ -1788,16 +1912,16 @@
           <t>ICU</t>
         </is>
       </c>
-      <c r="B3" s="10" t="n">
+      <c r="B3" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="C3" s="10" t="n">
+      <c r="C3" s="12" t="n">
         <v>0.5</v>
       </c>
-      <c r="D3" s="10" t="n">
+      <c r="D3" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="10" t="n">
+      <c r="E3" s="12" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1807,16 +1931,16 @@
           <t>Telemetry</t>
         </is>
       </c>
-      <c r="B4" s="10" t="n">
+      <c r="B4" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="C4" s="10" t="n">
+      <c r="C4" s="12" t="n">
         <v>0.55</v>
       </c>
-      <c r="D4" s="10" t="n">
+      <c r="D4" s="12" t="n">
         <v>0.7</v>
       </c>
-      <c r="E4" s="10" t="n">
+      <c r="E4" s="12" t="n">
         <v>0.65</v>
       </c>
     </row>
@@ -1865,42 +1989,42 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>OT_Threshold_Weekly_Hours</t>
         </is>
       </c>
-      <c r="B2" s="10" t="n">
+      <c r="B2" s="12" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Rest_Hours_Between_Shifts</t>
         </is>
       </c>
-      <c r="B3" s="10" t="n">
+      <c r="B3" s="12" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>Max_Consecutive_Days</t>
         </is>
       </c>
-      <c r="B4" s="10" t="n">
+      <c r="B4" s="12" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Shift_Basis_Hours</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="12" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1973,306 +2097,306 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>D12</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>Day 12hr</t>
         </is>
       </c>
-      <c r="C2" s="13" t="inlineStr">
+      <c r="C2" s="14" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="D2" s="13" t="n">
+      <c r="D2" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="E2" s="13" t="n">
+      <c r="E2" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="F2" s="13" t="n">
+      <c r="F2" s="14" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>D8</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Day 8hr</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="D3" s="13" t="n">
+      <c r="D3" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="E3" s="13" t="n">
+      <c r="E3" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="F3" s="13" t="n">
+      <c r="F3" s="14" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>E8</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Evening 8hr</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="D4" s="13" t="n">
+      <c r="D4" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="13" t="n">
+      <c r="E4" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="F4" s="13" t="n">
+      <c r="F4" s="14" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>P4D</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>Part-time 4hr day</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="F5" s="14" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>N12</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Night 12hr</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>Night</t>
         </is>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="E6" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="F6" s="13" t="n">
+      <c r="F6" s="14" t="n">
         <v>31</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>N8</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>Night 8hr</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>Night</t>
         </is>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="E7" s="13" t="n">
+      <c r="E7" s="14" t="n">
         <v>23</v>
       </c>
-      <c r="F7" s="13" t="n">
+      <c r="F7" s="14" t="n">
         <v>31</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>P4N</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>Part-time 4hr night</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>Night</t>
         </is>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="13" t="n">
+      <c r="E8" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="F8" s="13" t="n">
+      <c r="F8" s="14" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>PTO</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>Paid Time Off</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
       </c>
-      <c r="D9" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="13" t="n">
+      <c r="D9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>SICK</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>Sick Leave</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
       </c>
-      <c r="D10" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="13" t="n">
+      <c r="D10" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>VAC</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>Vacation</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
       </c>
-      <c r="D11" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="13" t="n">
+      <c r="D11" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>Work Off</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
       </c>
-      <c r="D12" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="13" t="n">
+      <c r="D12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="10" t="n"/>
+      <c r="A13" s="12" t="n"/>
+      <c r="B13" s="12" t="n"/>
+      <c r="C13" s="12" t="n"/>
+      <c r="D13" s="12" t="n"/>
+      <c r="E13" s="12" t="n"/>
+      <c r="F13" s="12" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
+      <c r="A14" s="12" t="n"/>
+      <c r="B14" s="12" t="n"/>
+      <c r="C14" s="12" t="n"/>
+      <c r="D14" s="12" t="n"/>
+      <c r="E14" s="12" t="n"/>
+      <c r="F14" s="12" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
@@ -2327,31 +2451,31 @@
           <t>Unit \ Date</t>
         </is>
       </c>
-      <c r="B1" s="15">
+      <c r="B1" s="16">
         <f>Schedule!D4</f>
         <v/>
       </c>
-      <c r="C1" s="15">
+      <c r="C1" s="16">
         <f>Schedule!E4</f>
         <v/>
       </c>
-      <c r="D1" s="15">
+      <c r="D1" s="16">
         <f>Schedule!F4</f>
         <v/>
       </c>
-      <c r="E1" s="15">
+      <c r="E1" s="16">
         <f>Schedule!G4</f>
         <v/>
       </c>
-      <c r="F1" s="15">
+      <c r="F1" s="16">
         <f>Schedule!H4</f>
         <v/>
       </c>
-      <c r="G1" s="15">
+      <c r="G1" s="16">
         <f>Schedule!I4</f>
         <v/>
       </c>
-      <c r="H1" s="15">
+      <c r="H1" s="16">
         <f>Schedule!J4</f>
         <v/>
       </c>
@@ -2362,83 +2486,83 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12">
+      <c r="A2" s="13">
         <f>Units!A2</f>
         <v/>
       </c>
-      <c r="B2" s="10" t="n">
+      <c r="B2" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="C2" s="10" t="n">
+      <c r="C2" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="D2" s="10" t="n">
+      <c r="D2" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="E2" s="10" t="n">
+      <c r="E2" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="F2" s="10" t="n">
+      <c r="F2" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="G2" s="10" t="n">
+      <c r="G2" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="H2" s="10" t="n">
+      <c r="H2" s="12" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12">
+      <c r="A3" s="13">
         <f>Units!A3</f>
         <v/>
       </c>
-      <c r="B3" s="10" t="n">
+      <c r="B3" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="C3" s="10" t="n">
+      <c r="C3" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="D3" s="10" t="n">
+      <c r="D3" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="E3" s="10" t="n">
+      <c r="E3" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="F3" s="10" t="n">
+      <c r="F3" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="G3" s="10" t="n">
+      <c r="G3" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="H3" s="10" t="n">
+      <c r="H3" s="12" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12">
+      <c r="A4" s="13">
         <f>Units!A4</f>
         <v/>
       </c>
-      <c r="B4" s="10" t="n">
+      <c r="B4" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="C4" s="10" t="n">
+      <c r="C4" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="D4" s="10" t="n">
+      <c r="D4" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="E4" s="10" t="n">
+      <c r="E4" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="F4" s="10" t="n">
+      <c r="F4" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="G4" s="10" t="n">
+      <c r="G4" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="H4" s="10" t="n">
+      <c r="H4" s="12" t="n">
         <v>16</v>
       </c>
     </row>
@@ -2487,86 +2611,86 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="n">
+      <c r="A2" s="17" t="n">
         <v>45967</v>
       </c>
-      <c r="B2" s="17" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>Public Holiday A</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="n"/>
-      <c r="B3" s="18" t="n"/>
+      <c r="A3" s="10" t="n"/>
+      <c r="B3" s="10" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="n"/>
-      <c r="B4" s="18" t="n"/>
+      <c r="A4" s="10" t="n"/>
+      <c r="B4" s="10" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="n"/>
-      <c r="B5" s="18" t="n"/>
+      <c r="A5" s="10" t="n"/>
+      <c r="B5" s="10" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="n"/>
-      <c r="B6" s="18" t="n"/>
+      <c r="A6" s="10" t="n"/>
+      <c r="B6" s="10" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="n"/>
-      <c r="B7" s="18" t="n"/>
+      <c r="A7" s="10" t="n"/>
+      <c r="B7" s="10" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="n"/>
-      <c r="B8" s="18" t="n"/>
+      <c r="A8" s="10" t="n"/>
+      <c r="B8" s="10" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="n"/>
-      <c r="B9" s="18" t="n"/>
+      <c r="A9" s="10" t="n"/>
+      <c r="B9" s="10" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="n"/>
-      <c r="B10" s="18" t="n"/>
+      <c r="A10" s="10" t="n"/>
+      <c r="B10" s="10" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="n"/>
-      <c r="B11" s="18" t="n"/>
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="n"/>
-      <c r="B12" s="18" t="n"/>
+      <c r="A12" s="10" t="n"/>
+      <c r="B12" s="10" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="n"/>
-      <c r="B13" s="18" t="n"/>
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="n"/>
-      <c r="B14" s="18" t="n"/>
+      <c r="A14" s="10" t="n"/>
+      <c r="B14" s="10" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="n"/>
-      <c r="B15" s="18" t="n"/>
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="10" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="n"/>
-      <c r="B16" s="18" t="n"/>
+      <c r="A16" s="10" t="n"/>
+      <c r="B16" s="10" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="18" t="n"/>
-      <c r="B17" s="18" t="n"/>
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="10" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="18" t="n"/>
-      <c r="B18" s="18" t="n"/>
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="10" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="18" t="n"/>
-      <c r="B19" s="18" t="n"/>
+      <c r="A19" s="10" t="n"/>
+      <c r="B19" s="10" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="n"/>
-      <c r="B20" s="18" t="n"/>
+      <c r="A20" s="10" t="n"/>
+      <c r="B20" s="10" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1" password="8610"/>
@@ -2623,13 +2747,13 @@
           <t>Smith, John</t>
         </is>
       </c>
-      <c r="B2" s="16" t="n">
+      <c r="B2" s="17" t="n">
         <v>45964</v>
       </c>
-      <c r="C2" s="16" t="n">
+      <c r="C2" s="17" t="n">
         <v>45965</v>
       </c>
-      <c r="D2" s="17" t="inlineStr">
+      <c r="D2" s="18" t="inlineStr">
         <is>
           <t>PTO</t>
         </is>
@@ -2641,13 +2765,13 @@
           <t>Johnson, Emily</t>
         </is>
       </c>
-      <c r="B3" s="16" t="n">
+      <c r="B3" s="17" t="n">
         <v>45966</v>
       </c>
-      <c r="C3" s="16" t="n">
+      <c r="C3" s="17" t="n">
         <v>45966</v>
       </c>
-      <c r="D3" s="17" t="inlineStr">
+      <c r="D3" s="18" t="inlineStr">
         <is>
           <t>SICK</t>
         </is>
@@ -2659,113 +2783,113 @@
           <t>Garcia, Sarah</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="17" t="n">
         <v>45969</v>
       </c>
-      <c r="C4" s="16" t="n">
+      <c r="C4" s="17" t="n">
         <v>45970</v>
       </c>
-      <c r="D4" s="17" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>VAC</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="n"/>
-      <c r="B5" s="18" t="n"/>
-      <c r="C5" s="18" t="n"/>
-      <c r="D5" s="18" t="n"/>
+      <c r="A5" s="10" t="n"/>
+      <c r="B5" s="10" t="n"/>
+      <c r="C5" s="10" t="n"/>
+      <c r="D5" s="10" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="n"/>
-      <c r="B6" s="18" t="n"/>
-      <c r="C6" s="18" t="n"/>
-      <c r="D6" s="18" t="n"/>
+      <c r="A6" s="10" t="n"/>
+      <c r="B6" s="10" t="n"/>
+      <c r="C6" s="10" t="n"/>
+      <c r="D6" s="10" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="n"/>
-      <c r="B7" s="18" t="n"/>
-      <c r="C7" s="18" t="n"/>
-      <c r="D7" s="18" t="n"/>
+      <c r="A7" s="10" t="n"/>
+      <c r="B7" s="10" t="n"/>
+      <c r="C7" s="10" t="n"/>
+      <c r="D7" s="10" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="n"/>
-      <c r="B8" s="18" t="n"/>
-      <c r="C8" s="18" t="n"/>
-      <c r="D8" s="18" t="n"/>
+      <c r="A8" s="10" t="n"/>
+      <c r="B8" s="10" t="n"/>
+      <c r="C8" s="10" t="n"/>
+      <c r="D8" s="10" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="n"/>
-      <c r="B9" s="18" t="n"/>
-      <c r="C9" s="18" t="n"/>
-      <c r="D9" s="18" t="n"/>
+      <c r="A9" s="10" t="n"/>
+      <c r="B9" s="10" t="n"/>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="10" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="n"/>
-      <c r="B10" s="18" t="n"/>
-      <c r="C10" s="18" t="n"/>
-      <c r="D10" s="18" t="n"/>
+      <c r="A10" s="10" t="n"/>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="n"/>
-      <c r="B11" s="18" t="n"/>
-      <c r="C11" s="18" t="n"/>
-      <c r="D11" s="18" t="n"/>
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="n"/>
-      <c r="B12" s="18" t="n"/>
-      <c r="C12" s="18" t="n"/>
-      <c r="D12" s="18" t="n"/>
+      <c r="A12" s="10" t="n"/>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="10" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="n"/>
-      <c r="B13" s="18" t="n"/>
-      <c r="C13" s="18" t="n"/>
-      <c r="D13" s="18" t="n"/>
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="n"/>
-      <c r="B14" s="18" t="n"/>
-      <c r="C14" s="18" t="n"/>
-      <c r="D14" s="18" t="n"/>
+      <c r="A14" s="10" t="n"/>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="10" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="n"/>
-      <c r="B15" s="18" t="n"/>
-      <c r="C15" s="18" t="n"/>
-      <c r="D15" s="18" t="n"/>
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="n"/>
-      <c r="B16" s="18" t="n"/>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="18" t="n"/>
+      <c r="A16" s="10" t="n"/>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="18" t="n"/>
-      <c r="B17" s="18" t="n"/>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="18" t="n"/>
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="18" t="n"/>
-      <c r="B18" s="18" t="n"/>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="18" t="n"/>
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="10" t="n"/>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="10" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="18" t="n"/>
-      <c r="B19" s="18" t="n"/>
-      <c r="C19" s="18" t="n"/>
-      <c r="D19" s="18" t="n"/>
+      <c r="A19" s="10" t="n"/>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="n"/>
-      <c r="B20" s="18" t="n"/>
-      <c r="C20" s="18" t="n"/>
-      <c r="D20" s="18" t="n"/>
+      <c r="A20" s="10" t="n"/>
+      <c r="B20" s="10" t="n"/>
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="10" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1" password="8610"/>
@@ -2780,11 +2904,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM36"/>
+  <dimension ref="A1:AM46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
@@ -2829,7 +2953,7 @@
           <t>Select Unit:</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Med-Surg</t>
         </is>
@@ -3126,12 +3250,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14">
-        <f>Staff!A2</f>
-        <v/>
-      </c>
-      <c r="B12" s="13">
-        <f>VLOOKUP(A12,StaffTbl,2,FALSE)</f>
+      <c r="A12" s="15">
+        <f>IF(Staff!A2="","",Staff!A2)</f>
+        <v/>
+      </c>
+      <c r="B12" s="14">
+        <f>IF(A12="","",VLOOKUP(A12,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D12" s="9" t="inlineStr">
@@ -3169,32 +3293,32 @@
           <t>N12</t>
         </is>
       </c>
-      <c r="K12" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D12:J12,ShiftHours))</f>
+      <c r="K12" s="14">
+        <f>IF($A12="","",SUMPRODUCT(SUMIF(ShiftCode,D12:J12,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L12" s="25">
-        <f>IF(K12&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M12" s="13">
-        <f>MAX(R12:X12)</f>
+        <f>IF($A12="","",IF(K12&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M12" s="14">
+        <f>IF($A12="","",MAX(R12:X12))</f>
         <v/>
       </c>
       <c r="N12" s="25">
-        <f>IF(M12&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O12" s="13">
-        <f>IF(MIN(Z12:AE12)=999,"",MIN(Z12:AE12))</f>
+        <f>IF($A12="","",IF(M12&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O12" s="14">
+        <f>IF($A12="","",IF(MIN(Z12:AE12)=999,"",MIN(Z12:AE12)))</f>
         <v/>
       </c>
       <c r="P12" s="25">
-        <f>IF(AND(O12&lt;&gt;"",O12&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A12="","",IF(AND(O12&lt;&gt;"",O12&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q12" s="25">
-        <f>IF(SUM(AG12:AM12)&gt;0,"CHECK","")</f>
+        <f>IF($A12="","",IF(SUM(AG12:AM12)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R12">
@@ -3279,12 +3403,12 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14">
-        <f>Staff!A3</f>
-        <v/>
-      </c>
-      <c r="B13" s="13">
-        <f>VLOOKUP(A13,StaffTbl,2,FALSE)</f>
+      <c r="A13" s="15">
+        <f>IF(Staff!A3="","",Staff!A3)</f>
+        <v/>
+      </c>
+      <c r="B13" s="14">
+        <f>IF(A13="","",VLOOKUP(A13,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D13" s="9" t="inlineStr">
@@ -3322,32 +3446,32 @@
           <t>N12</t>
         </is>
       </c>
-      <c r="K13" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D13:J13,ShiftHours))</f>
+      <c r="K13" s="14">
+        <f>IF($A13="","",SUMPRODUCT(SUMIF(ShiftCode,D13:J13,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L13" s="25">
-        <f>IF(K13&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M13" s="13">
-        <f>MAX(R13:X13)</f>
+        <f>IF($A13="","",IF(K13&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M13" s="14">
+        <f>IF($A13="","",MAX(R13:X13))</f>
         <v/>
       </c>
       <c r="N13" s="25">
-        <f>IF(M13&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O13" s="13">
-        <f>IF(MIN(Z13:AE13)=999,"",MIN(Z13:AE13))</f>
+        <f>IF($A13="","",IF(M13&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O13" s="14">
+        <f>IF($A13="","",IF(MIN(Z13:AE13)=999,"",MIN(Z13:AE13)))</f>
         <v/>
       </c>
       <c r="P13" s="25">
-        <f>IF(AND(O13&lt;&gt;"",O13&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A13="","",IF(AND(O13&lt;&gt;"",O13&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q13" s="25">
-        <f>IF(SUM(AG13:AM13)&gt;0,"CHECK","")</f>
+        <f>IF($A13="","",IF(SUM(AG13:AM13)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R13">
@@ -3432,12 +3556,12 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14">
-        <f>Staff!A4</f>
-        <v/>
-      </c>
-      <c r="B14" s="13">
-        <f>VLOOKUP(A14,StaffTbl,2,FALSE)</f>
+      <c r="A14" s="15">
+        <f>IF(Staff!A4="","",Staff!A4)</f>
+        <v/>
+      </c>
+      <c r="B14" s="14">
+        <f>IF(A14="","",VLOOKUP(A14,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D14" s="9" t="inlineStr">
@@ -3475,32 +3599,32 @@
           <t>D12</t>
         </is>
       </c>
-      <c r="K14" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D14:J14,ShiftHours))</f>
+      <c r="K14" s="14">
+        <f>IF($A14="","",SUMPRODUCT(SUMIF(ShiftCode,D14:J14,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L14" s="25">
-        <f>IF(K14&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M14" s="13">
-        <f>MAX(R14:X14)</f>
+        <f>IF($A14="","",IF(K14&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M14" s="14">
+        <f>IF($A14="","",MAX(R14:X14))</f>
         <v/>
       </c>
       <c r="N14" s="25">
-        <f>IF(M14&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O14" s="13">
-        <f>IF(MIN(Z14:AE14)=999,"",MIN(Z14:AE14))</f>
+        <f>IF($A14="","",IF(M14&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O14" s="14">
+        <f>IF($A14="","",IF(MIN(Z14:AE14)=999,"",MIN(Z14:AE14)))</f>
         <v/>
       </c>
       <c r="P14" s="25">
-        <f>IF(AND(O14&lt;&gt;"",O14&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A14="","",IF(AND(O14&lt;&gt;"",O14&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q14" s="25">
-        <f>IF(SUM(AG14:AM14)&gt;0,"CHECK","")</f>
+        <f>IF($A14="","",IF(SUM(AG14:AM14)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R14">
@@ -3585,12 +3709,12 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14">
-        <f>Staff!A5</f>
-        <v/>
-      </c>
-      <c r="B15" s="13">
-        <f>VLOOKUP(A15,StaffTbl,2,FALSE)</f>
+      <c r="A15" s="15">
+        <f>IF(Staff!A5="","",Staff!A5)</f>
+        <v/>
+      </c>
+      <c r="B15" s="14">
+        <f>IF(A15="","",VLOOKUP(A15,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D15" s="9" t="inlineStr">
@@ -3628,32 +3752,32 @@
           <t>D12</t>
         </is>
       </c>
-      <c r="K15" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D15:J15,ShiftHours))</f>
+      <c r="K15" s="14">
+        <f>IF($A15="","",SUMPRODUCT(SUMIF(ShiftCode,D15:J15,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L15" s="25">
-        <f>IF(K15&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M15" s="13">
-        <f>MAX(R15:X15)</f>
+        <f>IF($A15="","",IF(K15&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M15" s="14">
+        <f>IF($A15="","",MAX(R15:X15))</f>
         <v/>
       </c>
       <c r="N15" s="25">
-        <f>IF(M15&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O15" s="13">
-        <f>IF(MIN(Z15:AE15)=999,"",MIN(Z15:AE15))</f>
+        <f>IF($A15="","",IF(M15&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O15" s="14">
+        <f>IF($A15="","",IF(MIN(Z15:AE15)=999,"",MIN(Z15:AE15)))</f>
         <v/>
       </c>
       <c r="P15" s="25">
-        <f>IF(AND(O15&lt;&gt;"",O15&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A15="","",IF(AND(O15&lt;&gt;"",O15&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q15" s="25">
-        <f>IF(SUM(AG15:AM15)&gt;0,"CHECK","")</f>
+        <f>IF($A15="","",IF(SUM(AG15:AM15)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R15">
@@ -3738,12 +3862,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14">
-        <f>Staff!A6</f>
-        <v/>
-      </c>
-      <c r="B16" s="13">
-        <f>VLOOKUP(A16,StaffTbl,2,FALSE)</f>
+      <c r="A16" s="15">
+        <f>IF(Staff!A6="","",Staff!A6)</f>
+        <v/>
+      </c>
+      <c r="B16" s="14">
+        <f>IF(A16="","",VLOOKUP(A16,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D16" s="9" t="inlineStr">
@@ -3781,32 +3905,32 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="K16" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D16:J16,ShiftHours))</f>
+      <c r="K16" s="14">
+        <f>IF($A16="","",SUMPRODUCT(SUMIF(ShiftCode,D16:J16,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L16" s="25">
-        <f>IF(K16&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M16" s="13">
-        <f>MAX(R16:X16)</f>
+        <f>IF($A16="","",IF(K16&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M16" s="14">
+        <f>IF($A16="","",MAX(R16:X16))</f>
         <v/>
       </c>
       <c r="N16" s="25">
-        <f>IF(M16&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O16" s="13">
-        <f>IF(MIN(Z16:AE16)=999,"",MIN(Z16:AE16))</f>
+        <f>IF($A16="","",IF(M16&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O16" s="14">
+        <f>IF($A16="","",IF(MIN(Z16:AE16)=999,"",MIN(Z16:AE16)))</f>
         <v/>
       </c>
       <c r="P16" s="25">
-        <f>IF(AND(O16&lt;&gt;"",O16&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A16="","",IF(AND(O16&lt;&gt;"",O16&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q16" s="25">
-        <f>IF(SUM(AG16:AM16)&gt;0,"CHECK","")</f>
+        <f>IF($A16="","",IF(SUM(AG16:AM16)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R16">
@@ -3891,12 +4015,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="14">
-        <f>Staff!A7</f>
-        <v/>
-      </c>
-      <c r="B17" s="13">
-        <f>VLOOKUP(A17,StaffTbl,2,FALSE)</f>
+      <c r="A17" s="15">
+        <f>IF(Staff!A7="","",Staff!A7)</f>
+        <v/>
+      </c>
+      <c r="B17" s="14">
+        <f>IF(A17="","",VLOOKUP(A17,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D17" s="9" t="inlineStr">
@@ -3934,32 +4058,32 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="K17" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D17:J17,ShiftHours))</f>
+      <c r="K17" s="14">
+        <f>IF($A17="","",SUMPRODUCT(SUMIF(ShiftCode,D17:J17,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L17" s="25">
-        <f>IF(K17&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M17" s="13">
-        <f>MAX(R17:X17)</f>
+        <f>IF($A17="","",IF(K17&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M17" s="14">
+        <f>IF($A17="","",MAX(R17:X17))</f>
         <v/>
       </c>
       <c r="N17" s="25">
-        <f>IF(M17&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O17" s="13">
-        <f>IF(MIN(Z17:AE17)=999,"",MIN(Z17:AE17))</f>
+        <f>IF($A17="","",IF(M17&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O17" s="14">
+        <f>IF($A17="","",IF(MIN(Z17:AE17)=999,"",MIN(Z17:AE17)))</f>
         <v/>
       </c>
       <c r="P17" s="25">
-        <f>IF(AND(O17&lt;&gt;"",O17&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A17="","",IF(AND(O17&lt;&gt;"",O17&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q17" s="25">
-        <f>IF(SUM(AG17:AM17)&gt;0,"CHECK","")</f>
+        <f>IF($A17="","",IF(SUM(AG17:AM17)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R17">
@@ -4044,12 +4168,12 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14">
-        <f>Staff!A8</f>
-        <v/>
-      </c>
-      <c r="B18" s="13">
-        <f>VLOOKUP(A18,StaffTbl,2,FALSE)</f>
+      <c r="A18" s="15">
+        <f>IF(Staff!A8="","",Staff!A8)</f>
+        <v/>
+      </c>
+      <c r="B18" s="14">
+        <f>IF(A18="","",VLOOKUP(A18,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D18" s="9" t="inlineStr">
@@ -4087,32 +4211,32 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="K18" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D18:J18,ShiftHours))</f>
+      <c r="K18" s="14">
+        <f>IF($A18="","",SUMPRODUCT(SUMIF(ShiftCode,D18:J18,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L18" s="25">
-        <f>IF(K18&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M18" s="13">
-        <f>MAX(R18:X18)</f>
+        <f>IF($A18="","",IF(K18&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M18" s="14">
+        <f>IF($A18="","",MAX(R18:X18))</f>
         <v/>
       </c>
       <c r="N18" s="25">
-        <f>IF(M18&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O18" s="13">
-        <f>IF(MIN(Z18:AE18)=999,"",MIN(Z18:AE18))</f>
+        <f>IF($A18="","",IF(M18&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O18" s="14">
+        <f>IF($A18="","",IF(MIN(Z18:AE18)=999,"",MIN(Z18:AE18)))</f>
         <v/>
       </c>
       <c r="P18" s="25">
-        <f>IF(AND(O18&lt;&gt;"",O18&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A18="","",IF(AND(O18&lt;&gt;"",O18&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q18" s="25">
-        <f>IF(SUM(AG18:AM18)&gt;0,"CHECK","")</f>
+        <f>IF($A18="","",IF(SUM(AG18:AM18)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R18">
@@ -4197,12 +4321,12 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="14">
-        <f>Staff!A9</f>
-        <v/>
-      </c>
-      <c r="B19" s="13">
-        <f>VLOOKUP(A19,StaffTbl,2,FALSE)</f>
+      <c r="A19" s="15">
+        <f>IF(Staff!A9="","",Staff!A9)</f>
+        <v/>
+      </c>
+      <c r="B19" s="14">
+        <f>IF(A19="","",VLOOKUP(A19,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D19" s="9" t="inlineStr">
@@ -4240,32 +4364,32 @@
           <t>N12</t>
         </is>
       </c>
-      <c r="K19" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D19:J19,ShiftHours))</f>
+      <c r="K19" s="14">
+        <f>IF($A19="","",SUMPRODUCT(SUMIF(ShiftCode,D19:J19,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L19" s="25">
-        <f>IF(K19&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M19" s="13">
-        <f>MAX(R19:X19)</f>
+        <f>IF($A19="","",IF(K19&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M19" s="14">
+        <f>IF($A19="","",MAX(R19:X19))</f>
         <v/>
       </c>
       <c r="N19" s="25">
-        <f>IF(M19&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O19" s="13">
-        <f>IF(MIN(Z19:AE19)=999,"",MIN(Z19:AE19))</f>
+        <f>IF($A19="","",IF(M19&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O19" s="14">
+        <f>IF($A19="","",IF(MIN(Z19:AE19)=999,"",MIN(Z19:AE19)))</f>
         <v/>
       </c>
       <c r="P19" s="25">
-        <f>IF(AND(O19&lt;&gt;"",O19&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A19="","",IF(AND(O19&lt;&gt;"",O19&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q19" s="25">
-        <f>IF(SUM(AG19:AM19)&gt;0,"CHECK","")</f>
+        <f>IF($A19="","",IF(SUM(AG19:AM19)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R19">
@@ -4350,12 +4474,12 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="14">
-        <f>Staff!A10</f>
-        <v/>
-      </c>
-      <c r="B20" s="13">
-        <f>VLOOKUP(A20,StaffTbl,2,FALSE)</f>
+      <c r="A20" s="15">
+        <f>IF(Staff!A10="","",Staff!A10)</f>
+        <v/>
+      </c>
+      <c r="B20" s="14">
+        <f>IF(A20="","",VLOOKUP(A20,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D20" s="9" t="inlineStr">
@@ -4393,32 +4517,32 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="K20" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D20:J20,ShiftHours))</f>
+      <c r="K20" s="14">
+        <f>IF($A20="","",SUMPRODUCT(SUMIF(ShiftCode,D20:J20,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L20" s="25">
-        <f>IF(K20&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M20" s="13">
-        <f>MAX(R20:X20)</f>
+        <f>IF($A20="","",IF(K20&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M20" s="14">
+        <f>IF($A20="","",MAX(R20:X20))</f>
         <v/>
       </c>
       <c r="N20" s="25">
-        <f>IF(M20&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O20" s="13">
-        <f>IF(MIN(Z20:AE20)=999,"",MIN(Z20:AE20))</f>
+        <f>IF($A20="","",IF(M20&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O20" s="14">
+        <f>IF($A20="","",IF(MIN(Z20:AE20)=999,"",MIN(Z20:AE20)))</f>
         <v/>
       </c>
       <c r="P20" s="25">
-        <f>IF(AND(O20&lt;&gt;"",O20&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A20="","",IF(AND(O20&lt;&gt;"",O20&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q20" s="25">
-        <f>IF(SUM(AG20:AM20)&gt;0,"CHECK","")</f>
+        <f>IF($A20="","",IF(SUM(AG20:AM20)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R20">
@@ -4503,12 +4627,12 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="14">
-        <f>Staff!A11</f>
-        <v/>
-      </c>
-      <c r="B21" s="13">
-        <f>VLOOKUP(A21,StaffTbl,2,FALSE)</f>
+      <c r="A21" s="15">
+        <f>IF(Staff!A11="","",Staff!A11)</f>
+        <v/>
+      </c>
+      <c r="B21" s="14">
+        <f>IF(A21="","",VLOOKUP(A21,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D21" s="9" t="inlineStr">
@@ -4546,32 +4670,32 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="K21" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D21:J21,ShiftHours))</f>
+      <c r="K21" s="14">
+        <f>IF($A21="","",SUMPRODUCT(SUMIF(ShiftCode,D21:J21,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L21" s="25">
-        <f>IF(K21&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M21" s="13">
-        <f>MAX(R21:X21)</f>
+        <f>IF($A21="","",IF(K21&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M21" s="14">
+        <f>IF($A21="","",MAX(R21:X21))</f>
         <v/>
       </c>
       <c r="N21" s="25">
-        <f>IF(M21&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O21" s="13">
-        <f>IF(MIN(Z21:AE21)=999,"",MIN(Z21:AE21))</f>
+        <f>IF($A21="","",IF(M21&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O21" s="14">
+        <f>IF($A21="","",IF(MIN(Z21:AE21)=999,"",MIN(Z21:AE21)))</f>
         <v/>
       </c>
       <c r="P21" s="25">
-        <f>IF(AND(O21&lt;&gt;"",O21&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A21="","",IF(AND(O21&lt;&gt;"",O21&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q21" s="25">
-        <f>IF(SUM(AG21:AM21)&gt;0,"CHECK","")</f>
+        <f>IF($A21="","",IF(SUM(AG21:AM21)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R21">
@@ -4656,12 +4780,12 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="14">
-        <f>Staff!A12</f>
-        <v/>
-      </c>
-      <c r="B22" s="13">
-        <f>VLOOKUP(A22,StaffTbl,2,FALSE)</f>
+      <c r="A22" s="15">
+        <f>IF(Staff!A12="","",Staff!A12)</f>
+        <v/>
+      </c>
+      <c r="B22" s="14">
+        <f>IF(A22="","",VLOOKUP(A22,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D22" s="9" t="inlineStr">
@@ -4699,32 +4823,32 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="K22" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D22:J22,ShiftHours))</f>
+      <c r="K22" s="14">
+        <f>IF($A22="","",SUMPRODUCT(SUMIF(ShiftCode,D22:J22,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L22" s="25">
-        <f>IF(K22&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M22" s="13">
-        <f>MAX(R22:X22)</f>
+        <f>IF($A22="","",IF(K22&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M22" s="14">
+        <f>IF($A22="","",MAX(R22:X22))</f>
         <v/>
       </c>
       <c r="N22" s="25">
-        <f>IF(M22&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O22" s="13">
-        <f>IF(MIN(Z22:AE22)=999,"",MIN(Z22:AE22))</f>
+        <f>IF($A22="","",IF(M22&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O22" s="14">
+        <f>IF($A22="","",IF(MIN(Z22:AE22)=999,"",MIN(Z22:AE22)))</f>
         <v/>
       </c>
       <c r="P22" s="25">
-        <f>IF(AND(O22&lt;&gt;"",O22&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A22="","",IF(AND(O22&lt;&gt;"",O22&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q22" s="25">
-        <f>IF(SUM(AG22:AM22)&gt;0,"CHECK","")</f>
+        <f>IF($A22="","",IF(SUM(AG22:AM22)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R22">
@@ -4809,12 +4933,12 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="14">
-        <f>Staff!A13</f>
-        <v/>
-      </c>
-      <c r="B23" s="13">
-        <f>VLOOKUP(A23,StaffTbl,2,FALSE)</f>
+      <c r="A23" s="15">
+        <f>IF(Staff!A13="","",Staff!A13)</f>
+        <v/>
+      </c>
+      <c r="B23" s="14">
+        <f>IF(A23="","",VLOOKUP(A23,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D23" s="9" t="inlineStr">
@@ -4852,32 +4976,32 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="K23" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D23:J23,ShiftHours))</f>
+      <c r="K23" s="14">
+        <f>IF($A23="","",SUMPRODUCT(SUMIF(ShiftCode,D23:J23,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L23" s="25">
-        <f>IF(K23&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M23" s="13">
-        <f>MAX(R23:X23)</f>
+        <f>IF($A23="","",IF(K23&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M23" s="14">
+        <f>IF($A23="","",MAX(R23:X23))</f>
         <v/>
       </c>
       <c r="N23" s="25">
-        <f>IF(M23&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O23" s="13">
-        <f>IF(MIN(Z23:AE23)=999,"",MIN(Z23:AE23))</f>
+        <f>IF($A23="","",IF(M23&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O23" s="14">
+        <f>IF($A23="","",IF(MIN(Z23:AE23)=999,"",MIN(Z23:AE23)))</f>
         <v/>
       </c>
       <c r="P23" s="25">
-        <f>IF(AND(O23&lt;&gt;"",O23&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A23="","",IF(AND(O23&lt;&gt;"",O23&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q23" s="25">
-        <f>IF(SUM(AG23:AM23)&gt;0,"CHECK","")</f>
+        <f>IF($A23="","",IF(SUM(AG23:AM23)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R23">
@@ -4962,12 +5086,12 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="14">
-        <f>Staff!A14</f>
-        <v/>
-      </c>
-      <c r="B24" s="13">
-        <f>VLOOKUP(A24,StaffTbl,2,FALSE)</f>
+      <c r="A24" s="15">
+        <f>IF(Staff!A14="","",Staff!A14)</f>
+        <v/>
+      </c>
+      <c r="B24" s="14">
+        <f>IF(A24="","",VLOOKUP(A24,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D24" s="9" t="inlineStr">
@@ -5005,32 +5129,32 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="K24" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D24:J24,ShiftHours))</f>
+      <c r="K24" s="14">
+        <f>IF($A24="","",SUMPRODUCT(SUMIF(ShiftCode,D24:J24,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L24" s="25">
-        <f>IF(K24&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M24" s="13">
-        <f>MAX(R24:X24)</f>
+        <f>IF($A24="","",IF(K24&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M24" s="14">
+        <f>IF($A24="","",MAX(R24:X24))</f>
         <v/>
       </c>
       <c r="N24" s="25">
-        <f>IF(M24&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O24" s="13">
-        <f>IF(MIN(Z24:AE24)=999,"",MIN(Z24:AE24))</f>
+        <f>IF($A24="","",IF(M24&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O24" s="14">
+        <f>IF($A24="","",IF(MIN(Z24:AE24)=999,"",MIN(Z24:AE24)))</f>
         <v/>
       </c>
       <c r="P24" s="25">
-        <f>IF(AND(O24&lt;&gt;"",O24&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A24="","",IF(AND(O24&lt;&gt;"",O24&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q24" s="25">
-        <f>IF(SUM(AG24:AM24)&gt;0,"CHECK","")</f>
+        <f>IF($A24="","",IF(SUM(AG24:AM24)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R24">
@@ -5115,12 +5239,12 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="14">
-        <f>Staff!A15</f>
-        <v/>
-      </c>
-      <c r="B25" s="13">
-        <f>VLOOKUP(A25,StaffTbl,2,FALSE)</f>
+      <c r="A25" s="15">
+        <f>IF(Staff!A15="","",Staff!A15)</f>
+        <v/>
+      </c>
+      <c r="B25" s="14">
+        <f>IF(A25="","",VLOOKUP(A25,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D25" s="9" t="inlineStr">
@@ -5158,32 +5282,32 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="K25" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D25:J25,ShiftHours))</f>
+      <c r="K25" s="14">
+        <f>IF($A25="","",SUMPRODUCT(SUMIF(ShiftCode,D25:J25,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L25" s="25">
-        <f>IF(K25&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M25" s="13">
-        <f>MAX(R25:X25)</f>
+        <f>IF($A25="","",IF(K25&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M25" s="14">
+        <f>IF($A25="","",MAX(R25:X25))</f>
         <v/>
       </c>
       <c r="N25" s="25">
-        <f>IF(M25&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O25" s="13">
-        <f>IF(MIN(Z25:AE25)=999,"",MIN(Z25:AE25))</f>
+        <f>IF($A25="","",IF(M25&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O25" s="14">
+        <f>IF($A25="","",IF(MIN(Z25:AE25)=999,"",MIN(Z25:AE25)))</f>
         <v/>
       </c>
       <c r="P25" s="25">
-        <f>IF(AND(O25&lt;&gt;"",O25&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A25="","",IF(AND(O25&lt;&gt;"",O25&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q25" s="25">
-        <f>IF(SUM(AG25:AM25)&gt;0,"CHECK","")</f>
+        <f>IF($A25="","",IF(SUM(AG25:AM25)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R25">
@@ -5268,12 +5392,12 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="14">
-        <f>Staff!A16</f>
-        <v/>
-      </c>
-      <c r="B26" s="13">
-        <f>VLOOKUP(A26,StaffTbl,2,FALSE)</f>
+      <c r="A26" s="15">
+        <f>IF(Staff!A16="","",Staff!A16)</f>
+        <v/>
+      </c>
+      <c r="B26" s="14">
+        <f>IF(A26="","",VLOOKUP(A26,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D26" s="9" t="inlineStr">
@@ -5311,32 +5435,32 @@
           <t>D12</t>
         </is>
       </c>
-      <c r="K26" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D26:J26,ShiftHours))</f>
+      <c r="K26" s="14">
+        <f>IF($A26="","",SUMPRODUCT(SUMIF(ShiftCode,D26:J26,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L26" s="25">
-        <f>IF(K26&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M26" s="13">
-        <f>MAX(R26:X26)</f>
+        <f>IF($A26="","",IF(K26&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M26" s="14">
+        <f>IF($A26="","",MAX(R26:X26))</f>
         <v/>
       </c>
       <c r="N26" s="25">
-        <f>IF(M26&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O26" s="13">
-        <f>IF(MIN(Z26:AE26)=999,"",MIN(Z26:AE26))</f>
+        <f>IF($A26="","",IF(M26&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O26" s="14">
+        <f>IF($A26="","",IF(MIN(Z26:AE26)=999,"",MIN(Z26:AE26)))</f>
         <v/>
       </c>
       <c r="P26" s="25">
-        <f>IF(AND(O26&lt;&gt;"",O26&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A26="","",IF(AND(O26&lt;&gt;"",O26&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q26" s="25">
-        <f>IF(SUM(AG26:AM26)&gt;0,"CHECK","")</f>
+        <f>IF($A26="","",IF(SUM(AG26:AM26)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R26">
@@ -5421,12 +5545,12 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="14">
-        <f>Staff!A17</f>
-        <v/>
-      </c>
-      <c r="B27" s="13">
-        <f>VLOOKUP(A27,StaffTbl,2,FALSE)</f>
+      <c r="A27" s="15">
+        <f>IF(Staff!A17="","",Staff!A17)</f>
+        <v/>
+      </c>
+      <c r="B27" s="14">
+        <f>IF(A27="","",VLOOKUP(A27,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D27" s="9" t="inlineStr">
@@ -5464,32 +5588,32 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="K27" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D27:J27,ShiftHours))</f>
+      <c r="K27" s="14">
+        <f>IF($A27="","",SUMPRODUCT(SUMIF(ShiftCode,D27:J27,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L27" s="25">
-        <f>IF(K27&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M27" s="13">
-        <f>MAX(R27:X27)</f>
+        <f>IF($A27="","",IF(K27&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M27" s="14">
+        <f>IF($A27="","",MAX(R27:X27))</f>
         <v/>
       </c>
       <c r="N27" s="25">
-        <f>IF(M27&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O27" s="13">
-        <f>IF(MIN(Z27:AE27)=999,"",MIN(Z27:AE27))</f>
+        <f>IF($A27="","",IF(M27&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O27" s="14">
+        <f>IF($A27="","",IF(MIN(Z27:AE27)=999,"",MIN(Z27:AE27)))</f>
         <v/>
       </c>
       <c r="P27" s="25">
-        <f>IF(AND(O27&lt;&gt;"",O27&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A27="","",IF(AND(O27&lt;&gt;"",O27&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q27" s="25">
-        <f>IF(SUM(AG27:AM27)&gt;0,"CHECK","")</f>
+        <f>IF($A27="","",IF(SUM(AG27:AM27)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R27">
@@ -5574,12 +5698,12 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="14">
-        <f>Staff!A18</f>
-        <v/>
-      </c>
-      <c r="B28" s="13">
-        <f>VLOOKUP(A28,StaffTbl,2,FALSE)</f>
+      <c r="A28" s="15">
+        <f>IF(Staff!A18="","",Staff!A18)</f>
+        <v/>
+      </c>
+      <c r="B28" s="14">
+        <f>IF(A28="","",VLOOKUP(A28,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D28" s="9" t="inlineStr">
@@ -5617,32 +5741,32 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="K28" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D28:J28,ShiftHours))</f>
+      <c r="K28" s="14">
+        <f>IF($A28="","",SUMPRODUCT(SUMIF(ShiftCode,D28:J28,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L28" s="25">
-        <f>IF(K28&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M28" s="13">
-        <f>MAX(R28:X28)</f>
+        <f>IF($A28="","",IF(K28&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M28" s="14">
+        <f>IF($A28="","",MAX(R28:X28))</f>
         <v/>
       </c>
       <c r="N28" s="25">
-        <f>IF(M28&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O28" s="13">
-        <f>IF(MIN(Z28:AE28)=999,"",MIN(Z28:AE28))</f>
+        <f>IF($A28="","",IF(M28&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O28" s="14">
+        <f>IF($A28="","",IF(MIN(Z28:AE28)=999,"",MIN(Z28:AE28)))</f>
         <v/>
       </c>
       <c r="P28" s="25">
-        <f>IF(AND(O28&lt;&gt;"",O28&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A28="","",IF(AND(O28&lt;&gt;"",O28&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q28" s="25">
-        <f>IF(SUM(AG28:AM28)&gt;0,"CHECK","")</f>
+        <f>IF($A28="","",IF(SUM(AG28:AM28)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R28">
@@ -5727,12 +5851,12 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="14">
-        <f>Staff!A19</f>
-        <v/>
-      </c>
-      <c r="B29" s="13">
-        <f>VLOOKUP(A29,StaffTbl,2,FALSE)</f>
+      <c r="A29" s="15">
+        <f>IF(Staff!A19="","",Staff!A19)</f>
+        <v/>
+      </c>
+      <c r="B29" s="14">
+        <f>IF(A29="","",VLOOKUP(A29,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D29" s="9" t="inlineStr">
@@ -5770,32 +5894,32 @@
           <t>D12</t>
         </is>
       </c>
-      <c r="K29" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D29:J29,ShiftHours))</f>
+      <c r="K29" s="14">
+        <f>IF($A29="","",SUMPRODUCT(SUMIF(ShiftCode,D29:J29,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L29" s="25">
-        <f>IF(K29&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M29" s="13">
-        <f>MAX(R29:X29)</f>
+        <f>IF($A29="","",IF(K29&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M29" s="14">
+        <f>IF($A29="","",MAX(R29:X29))</f>
         <v/>
       </c>
       <c r="N29" s="25">
-        <f>IF(M29&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O29" s="13">
-        <f>IF(MIN(Z29:AE29)=999,"",MIN(Z29:AE29))</f>
+        <f>IF($A29="","",IF(M29&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O29" s="14">
+        <f>IF($A29="","",IF(MIN(Z29:AE29)=999,"",MIN(Z29:AE29)))</f>
         <v/>
       </c>
       <c r="P29" s="25">
-        <f>IF(AND(O29&lt;&gt;"",O29&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A29="","",IF(AND(O29&lt;&gt;"",O29&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q29" s="25">
-        <f>IF(SUM(AG29:AM29)&gt;0,"CHECK","")</f>
+        <f>IF($A29="","",IF(SUM(AG29:AM29)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R29">
@@ -5880,12 +6004,12 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="14">
-        <f>Staff!A20</f>
-        <v/>
-      </c>
-      <c r="B30" s="13">
-        <f>VLOOKUP(A30,StaffTbl,2,FALSE)</f>
+      <c r="A30" s="15">
+        <f>IF(Staff!A20="","",Staff!A20)</f>
+        <v/>
+      </c>
+      <c r="B30" s="14">
+        <f>IF(A30="","",VLOOKUP(A30,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D30" s="9" t="inlineStr">
@@ -5923,32 +6047,32 @@
           <t>D12</t>
         </is>
       </c>
-      <c r="K30" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D30:J30,ShiftHours))</f>
+      <c r="K30" s="14">
+        <f>IF($A30="","",SUMPRODUCT(SUMIF(ShiftCode,D30:J30,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L30" s="25">
-        <f>IF(K30&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M30" s="13">
-        <f>MAX(R30:X30)</f>
+        <f>IF($A30="","",IF(K30&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M30" s="14">
+        <f>IF($A30="","",MAX(R30:X30))</f>
         <v/>
       </c>
       <c r="N30" s="25">
-        <f>IF(M30&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O30" s="13">
-        <f>IF(MIN(Z30:AE30)=999,"",MIN(Z30:AE30))</f>
+        <f>IF($A30="","",IF(M30&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O30" s="14">
+        <f>IF($A30="","",IF(MIN(Z30:AE30)=999,"",MIN(Z30:AE30)))</f>
         <v/>
       </c>
       <c r="P30" s="25">
-        <f>IF(AND(O30&lt;&gt;"",O30&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A30="","",IF(AND(O30&lt;&gt;"",O30&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q30" s="25">
-        <f>IF(SUM(AG30:AM30)&gt;0,"CHECK","")</f>
+        <f>IF($A30="","",IF(SUM(AG30:AM30)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R30">
@@ -6033,12 +6157,12 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="14">
-        <f>Staff!A21</f>
-        <v/>
-      </c>
-      <c r="B31" s="13">
-        <f>VLOOKUP(A31,StaffTbl,2,FALSE)</f>
+      <c r="A31" s="15">
+        <f>IF(Staff!A21="","",Staff!A21)</f>
+        <v/>
+      </c>
+      <c r="B31" s="14">
+        <f>IF(A31="","",VLOOKUP(A31,StaffTbl,2,FALSE))</f>
         <v/>
       </c>
       <c r="D31" s="9" t="inlineStr">
@@ -6076,32 +6200,32 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="K31" s="13">
-        <f>SUMPRODUCT(SUMIF(ShiftCode,D31:J31,ShiftHours))</f>
+      <c r="K31" s="14">
+        <f>IF($A31="","",SUMPRODUCT(SUMIF(ShiftCode,D31:J31,ShiftHours)))</f>
         <v/>
       </c>
       <c r="L31" s="25">
-        <f>IF(K31&gt;OT_Threshold,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="M31" s="13">
-        <f>MAX(R31:X31)</f>
+        <f>IF($A31="","",IF(K31&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M31" s="14">
+        <f>IF($A31="","",MAX(R31:X31))</f>
         <v/>
       </c>
       <c r="N31" s="25">
-        <f>IF(M31&gt;Max_Consecutive,"OVER","")</f>
-        <v/>
-      </c>
-      <c r="O31" s="13">
-        <f>IF(MIN(Z31:AE31)=999,"",MIN(Z31:AE31))</f>
+        <f>IF($A31="","",IF(M31&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O31" s="14">
+        <f>IF($A31="","",IF(MIN(Z31:AE31)=999,"",MIN(Z31:AE31)))</f>
         <v/>
       </c>
       <c r="P31" s="25">
-        <f>IF(AND(O31&lt;&gt;"",O31&lt;Rest_Hours),"SHORT","")</f>
+        <f>IF($A31="","",IF(AND(O31&lt;&gt;"",O31&lt;Rest_Hours),"SHORT",""))</f>
         <v/>
       </c>
       <c r="Q31" s="25">
-        <f>IF(SUM(AG31:AM31)&gt;0,"CHECK","")</f>
+        <f>IF($A31="","",IF(SUM(AG31:AM31)&gt;0,"CHECK",""))</f>
         <v/>
       </c>
       <c r="R31">
@@ -6185,149 +6309,1399 @@
         <v/>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="15">
+        <f>IF(Staff!A22="","",Staff!A22)</f>
+        <v/>
+      </c>
+      <c r="B32" s="14">
+        <f>IF(A32="","",VLOOKUP(A32,StaffTbl,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D32" s="9" t="n"/>
+      <c r="E32" s="9" t="n"/>
+      <c r="F32" s="9" t="n"/>
+      <c r="G32" s="9" t="n"/>
+      <c r="H32" s="9" t="n"/>
+      <c r="I32" s="9" t="n"/>
+      <c r="J32" s="9" t="n"/>
+      <c r="K32" s="14">
+        <f>IF($A32="","",SUMPRODUCT(SUMIF(ShiftCode,D32:J32,ShiftHours)))</f>
+        <v/>
+      </c>
+      <c r="L32" s="25">
+        <f>IF($A32="","",IF(K32&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M32" s="14">
+        <f>IF($A32="","",MAX(R32:X32))</f>
+        <v/>
+      </c>
+      <c r="N32" s="25">
+        <f>IF($A32="","",IF(M32&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O32" s="14">
+        <f>IF($A32="","",IF(MIN(Z32:AE32)=999,"",MIN(Z32:AE32)))</f>
+        <v/>
+      </c>
+      <c r="P32" s="25">
+        <f>IF($A32="","",IF(AND(O32&lt;&gt;"",O32&lt;Rest_Hours),"SHORT",""))</f>
+        <v/>
+      </c>
+      <c r="Q32" s="25">
+        <f>IF($A32="","",IF(SUM(AG32:AM32)&gt;0,"CHECK",""))</f>
+        <v/>
+      </c>
+      <c r="R32">
+        <f>IF(SUMIF(ShiftCode,D32,ShiftHours)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="S32">
+        <f>IF(SUMIF(ShiftCode,E32,ShiftHours)&gt;0,R32+1,0)</f>
+        <v/>
+      </c>
+      <c r="T32">
+        <f>IF(SUMIF(ShiftCode,F32,ShiftHours)&gt;0,S32+1,0)</f>
+        <v/>
+      </c>
+      <c r="U32">
+        <f>IF(SUMIF(ShiftCode,G32,ShiftHours)&gt;0,T32+1,0)</f>
+        <v/>
+      </c>
+      <c r="V32">
+        <f>IF(SUMIF(ShiftCode,H32,ShiftHours)&gt;0,U32+1,0)</f>
+        <v/>
+      </c>
+      <c r="W32">
+        <f>IF(SUMIF(ShiftCode,I32,ShiftHours)&gt;0,V32+1,0)</f>
+        <v/>
+      </c>
+      <c r="X32">
+        <f>IF(SUMIF(ShiftCode,J32,ShiftHours)&gt;0,W32+1,0)</f>
+        <v/>
+      </c>
+      <c r="Z32">
+        <f>IF(AND(SUMIF(ShiftCode,D32,ShiftHours)&gt;0,SUMIF(ShiftCode,E32,ShiftHours)&gt;0),24+VLOOKUP(E32,ShiftFull,5,FALSE)-VLOOKUP(D32,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AA32">
+        <f>IF(AND(SUMIF(ShiftCode,E32,ShiftHours)&gt;0,SUMIF(ShiftCode,F32,ShiftHours)&gt;0),24+VLOOKUP(F32,ShiftFull,5,FALSE)-VLOOKUP(E32,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AB32">
+        <f>IF(AND(SUMIF(ShiftCode,F32,ShiftHours)&gt;0,SUMIF(ShiftCode,G32,ShiftHours)&gt;0),24+VLOOKUP(G32,ShiftFull,5,FALSE)-VLOOKUP(F32,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AC32">
+        <f>IF(AND(SUMIF(ShiftCode,G32,ShiftHours)&gt;0,SUMIF(ShiftCode,H32,ShiftHours)&gt;0),24+VLOOKUP(H32,ShiftFull,5,FALSE)-VLOOKUP(G32,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AD32">
+        <f>IF(AND(SUMIF(ShiftCode,H32,ShiftHours)&gt;0,SUMIF(ShiftCode,I32,ShiftHours)&gt;0),24+VLOOKUP(I32,ShiftFull,5,FALSE)-VLOOKUP(H32,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AE32">
+        <f>IF(AND(SUMIF(ShiftCode,I32,ShiftHours)&gt;0,SUMIF(ShiftCode,J32,ShiftHours)&gt;0),24+VLOOKUP(J32,ShiftFull,5,FALSE)-VLOOKUP(I32,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AG32">
+        <f>IF(AND(SUMIF(ShiftCode,D32,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A32)*(Leave!$B$2:$B$20&lt;=D$4)*(Leave!$C$2:$C$20&gt;=D$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AH32">
+        <f>IF(AND(SUMIF(ShiftCode,E32,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A32)*(Leave!$B$2:$B$20&lt;=E$4)*(Leave!$C$2:$C$20&gt;=E$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AI32">
+        <f>IF(AND(SUMIF(ShiftCode,F32,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A32)*(Leave!$B$2:$B$20&lt;=F$4)*(Leave!$C$2:$C$20&gt;=F$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AJ32">
+        <f>IF(AND(SUMIF(ShiftCode,G32,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A32)*(Leave!$B$2:$B$20&lt;=G$4)*(Leave!$C$2:$C$20&gt;=G$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AK32">
+        <f>IF(AND(SUMIF(ShiftCode,H32,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A32)*(Leave!$B$2:$B$20&lt;=H$4)*(Leave!$C$2:$C$20&gt;=H$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AL32">
+        <f>IF(AND(SUMIF(ShiftCode,I32,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A32)*(Leave!$B$2:$B$20&lt;=I$4)*(Leave!$C$2:$C$20&gt;=I$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AM32">
+        <f>IF(AND(SUMIF(ShiftCode,J32,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A32)*(Leave!$B$2:$B$20&lt;=J$4)*(Leave!$C$2:$C$20&gt;=J$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+    </row>
     <row r="33">
-      <c r="A33" s="20" t="inlineStr">
+      <c r="A33" s="15">
+        <f>IF(Staff!A23="","",Staff!A23)</f>
+        <v/>
+      </c>
+      <c r="B33" s="14">
+        <f>IF(A33="","",VLOOKUP(A33,StaffTbl,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D33" s="9" t="n"/>
+      <c r="E33" s="9" t="n"/>
+      <c r="F33" s="9" t="n"/>
+      <c r="G33" s="9" t="n"/>
+      <c r="H33" s="9" t="n"/>
+      <c r="I33" s="9" t="n"/>
+      <c r="J33" s="9" t="n"/>
+      <c r="K33" s="14">
+        <f>IF($A33="","",SUMPRODUCT(SUMIF(ShiftCode,D33:J33,ShiftHours)))</f>
+        <v/>
+      </c>
+      <c r="L33" s="25">
+        <f>IF($A33="","",IF(K33&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M33" s="14">
+        <f>IF($A33="","",MAX(R33:X33))</f>
+        <v/>
+      </c>
+      <c r="N33" s="25">
+        <f>IF($A33="","",IF(M33&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O33" s="14">
+        <f>IF($A33="","",IF(MIN(Z33:AE33)=999,"",MIN(Z33:AE33)))</f>
+        <v/>
+      </c>
+      <c r="P33" s="25">
+        <f>IF($A33="","",IF(AND(O33&lt;&gt;"",O33&lt;Rest_Hours),"SHORT",""))</f>
+        <v/>
+      </c>
+      <c r="Q33" s="25">
+        <f>IF($A33="","",IF(SUM(AG33:AM33)&gt;0,"CHECK",""))</f>
+        <v/>
+      </c>
+      <c r="R33">
+        <f>IF(SUMIF(ShiftCode,D33,ShiftHours)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="S33">
+        <f>IF(SUMIF(ShiftCode,E33,ShiftHours)&gt;0,R33+1,0)</f>
+        <v/>
+      </c>
+      <c r="T33">
+        <f>IF(SUMIF(ShiftCode,F33,ShiftHours)&gt;0,S33+1,0)</f>
+        <v/>
+      </c>
+      <c r="U33">
+        <f>IF(SUMIF(ShiftCode,G33,ShiftHours)&gt;0,T33+1,0)</f>
+        <v/>
+      </c>
+      <c r="V33">
+        <f>IF(SUMIF(ShiftCode,H33,ShiftHours)&gt;0,U33+1,0)</f>
+        <v/>
+      </c>
+      <c r="W33">
+        <f>IF(SUMIF(ShiftCode,I33,ShiftHours)&gt;0,V33+1,0)</f>
+        <v/>
+      </c>
+      <c r="X33">
+        <f>IF(SUMIF(ShiftCode,J33,ShiftHours)&gt;0,W33+1,0)</f>
+        <v/>
+      </c>
+      <c r="Z33">
+        <f>IF(AND(SUMIF(ShiftCode,D33,ShiftHours)&gt;0,SUMIF(ShiftCode,E33,ShiftHours)&gt;0),24+VLOOKUP(E33,ShiftFull,5,FALSE)-VLOOKUP(D33,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AA33">
+        <f>IF(AND(SUMIF(ShiftCode,E33,ShiftHours)&gt;0,SUMIF(ShiftCode,F33,ShiftHours)&gt;0),24+VLOOKUP(F33,ShiftFull,5,FALSE)-VLOOKUP(E33,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AB33">
+        <f>IF(AND(SUMIF(ShiftCode,F33,ShiftHours)&gt;0,SUMIF(ShiftCode,G33,ShiftHours)&gt;0),24+VLOOKUP(G33,ShiftFull,5,FALSE)-VLOOKUP(F33,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AC33">
+        <f>IF(AND(SUMIF(ShiftCode,G33,ShiftHours)&gt;0,SUMIF(ShiftCode,H33,ShiftHours)&gt;0),24+VLOOKUP(H33,ShiftFull,5,FALSE)-VLOOKUP(G33,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AD33">
+        <f>IF(AND(SUMIF(ShiftCode,H33,ShiftHours)&gt;0,SUMIF(ShiftCode,I33,ShiftHours)&gt;0),24+VLOOKUP(I33,ShiftFull,5,FALSE)-VLOOKUP(H33,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AE33">
+        <f>IF(AND(SUMIF(ShiftCode,I33,ShiftHours)&gt;0,SUMIF(ShiftCode,J33,ShiftHours)&gt;0),24+VLOOKUP(J33,ShiftFull,5,FALSE)-VLOOKUP(I33,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AG33">
+        <f>IF(AND(SUMIF(ShiftCode,D33,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A33)*(Leave!$B$2:$B$20&lt;=D$4)*(Leave!$C$2:$C$20&gt;=D$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AH33">
+        <f>IF(AND(SUMIF(ShiftCode,E33,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A33)*(Leave!$B$2:$B$20&lt;=E$4)*(Leave!$C$2:$C$20&gt;=E$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AI33">
+        <f>IF(AND(SUMIF(ShiftCode,F33,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A33)*(Leave!$B$2:$B$20&lt;=F$4)*(Leave!$C$2:$C$20&gt;=F$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AJ33">
+        <f>IF(AND(SUMIF(ShiftCode,G33,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A33)*(Leave!$B$2:$B$20&lt;=G$4)*(Leave!$C$2:$C$20&gt;=G$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AK33">
+        <f>IF(AND(SUMIF(ShiftCode,H33,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A33)*(Leave!$B$2:$B$20&lt;=H$4)*(Leave!$C$2:$C$20&gt;=H$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AL33">
+        <f>IF(AND(SUMIF(ShiftCode,I33,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A33)*(Leave!$B$2:$B$20&lt;=I$4)*(Leave!$C$2:$C$20&gt;=I$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AM33">
+        <f>IF(AND(SUMIF(ShiftCode,J33,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A33)*(Leave!$B$2:$B$20&lt;=J$4)*(Leave!$C$2:$C$20&gt;=J$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="15">
+        <f>IF(Staff!A24="","",Staff!A24)</f>
+        <v/>
+      </c>
+      <c r="B34" s="14">
+        <f>IF(A34="","",VLOOKUP(A34,StaffTbl,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D34" s="9" t="n"/>
+      <c r="E34" s="9" t="n"/>
+      <c r="F34" s="9" t="n"/>
+      <c r="G34" s="9" t="n"/>
+      <c r="H34" s="9" t="n"/>
+      <c r="I34" s="9" t="n"/>
+      <c r="J34" s="9" t="n"/>
+      <c r="K34" s="14">
+        <f>IF($A34="","",SUMPRODUCT(SUMIF(ShiftCode,D34:J34,ShiftHours)))</f>
+        <v/>
+      </c>
+      <c r="L34" s="25">
+        <f>IF($A34="","",IF(K34&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M34" s="14">
+        <f>IF($A34="","",MAX(R34:X34))</f>
+        <v/>
+      </c>
+      <c r="N34" s="25">
+        <f>IF($A34="","",IF(M34&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O34" s="14">
+        <f>IF($A34="","",IF(MIN(Z34:AE34)=999,"",MIN(Z34:AE34)))</f>
+        <v/>
+      </c>
+      <c r="P34" s="25">
+        <f>IF($A34="","",IF(AND(O34&lt;&gt;"",O34&lt;Rest_Hours),"SHORT",""))</f>
+        <v/>
+      </c>
+      <c r="Q34" s="25">
+        <f>IF($A34="","",IF(SUM(AG34:AM34)&gt;0,"CHECK",""))</f>
+        <v/>
+      </c>
+      <c r="R34">
+        <f>IF(SUMIF(ShiftCode,D34,ShiftHours)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="S34">
+        <f>IF(SUMIF(ShiftCode,E34,ShiftHours)&gt;0,R34+1,0)</f>
+        <v/>
+      </c>
+      <c r="T34">
+        <f>IF(SUMIF(ShiftCode,F34,ShiftHours)&gt;0,S34+1,0)</f>
+        <v/>
+      </c>
+      <c r="U34">
+        <f>IF(SUMIF(ShiftCode,G34,ShiftHours)&gt;0,T34+1,0)</f>
+        <v/>
+      </c>
+      <c r="V34">
+        <f>IF(SUMIF(ShiftCode,H34,ShiftHours)&gt;0,U34+1,0)</f>
+        <v/>
+      </c>
+      <c r="W34">
+        <f>IF(SUMIF(ShiftCode,I34,ShiftHours)&gt;0,V34+1,0)</f>
+        <v/>
+      </c>
+      <c r="X34">
+        <f>IF(SUMIF(ShiftCode,J34,ShiftHours)&gt;0,W34+1,0)</f>
+        <v/>
+      </c>
+      <c r="Z34">
+        <f>IF(AND(SUMIF(ShiftCode,D34,ShiftHours)&gt;0,SUMIF(ShiftCode,E34,ShiftHours)&gt;0),24+VLOOKUP(E34,ShiftFull,5,FALSE)-VLOOKUP(D34,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AA34">
+        <f>IF(AND(SUMIF(ShiftCode,E34,ShiftHours)&gt;0,SUMIF(ShiftCode,F34,ShiftHours)&gt;0),24+VLOOKUP(F34,ShiftFull,5,FALSE)-VLOOKUP(E34,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AB34">
+        <f>IF(AND(SUMIF(ShiftCode,F34,ShiftHours)&gt;0,SUMIF(ShiftCode,G34,ShiftHours)&gt;0),24+VLOOKUP(G34,ShiftFull,5,FALSE)-VLOOKUP(F34,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AC34">
+        <f>IF(AND(SUMIF(ShiftCode,G34,ShiftHours)&gt;0,SUMIF(ShiftCode,H34,ShiftHours)&gt;0),24+VLOOKUP(H34,ShiftFull,5,FALSE)-VLOOKUP(G34,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AD34">
+        <f>IF(AND(SUMIF(ShiftCode,H34,ShiftHours)&gt;0,SUMIF(ShiftCode,I34,ShiftHours)&gt;0),24+VLOOKUP(I34,ShiftFull,5,FALSE)-VLOOKUP(H34,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AE34">
+        <f>IF(AND(SUMIF(ShiftCode,I34,ShiftHours)&gt;0,SUMIF(ShiftCode,J34,ShiftHours)&gt;0),24+VLOOKUP(J34,ShiftFull,5,FALSE)-VLOOKUP(I34,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AG34">
+        <f>IF(AND(SUMIF(ShiftCode,D34,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A34)*(Leave!$B$2:$B$20&lt;=D$4)*(Leave!$C$2:$C$20&gt;=D$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AH34">
+        <f>IF(AND(SUMIF(ShiftCode,E34,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A34)*(Leave!$B$2:$B$20&lt;=E$4)*(Leave!$C$2:$C$20&gt;=E$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AI34">
+        <f>IF(AND(SUMIF(ShiftCode,F34,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A34)*(Leave!$B$2:$B$20&lt;=F$4)*(Leave!$C$2:$C$20&gt;=F$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AJ34">
+        <f>IF(AND(SUMIF(ShiftCode,G34,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A34)*(Leave!$B$2:$B$20&lt;=G$4)*(Leave!$C$2:$C$20&gt;=G$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AK34">
+        <f>IF(AND(SUMIF(ShiftCode,H34,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A34)*(Leave!$B$2:$B$20&lt;=H$4)*(Leave!$C$2:$C$20&gt;=H$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AL34">
+        <f>IF(AND(SUMIF(ShiftCode,I34,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A34)*(Leave!$B$2:$B$20&lt;=I$4)*(Leave!$C$2:$C$20&gt;=I$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AM34">
+        <f>IF(AND(SUMIF(ShiftCode,J34,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A34)*(Leave!$B$2:$B$20&lt;=J$4)*(Leave!$C$2:$C$20&gt;=J$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="15">
+        <f>IF(Staff!A25="","",Staff!A25)</f>
+        <v/>
+      </c>
+      <c r="B35" s="14">
+        <f>IF(A35="","",VLOOKUP(A35,StaffTbl,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D35" s="9" t="n"/>
+      <c r="E35" s="9" t="n"/>
+      <c r="F35" s="9" t="n"/>
+      <c r="G35" s="9" t="n"/>
+      <c r="H35" s="9" t="n"/>
+      <c r="I35" s="9" t="n"/>
+      <c r="J35" s="9" t="n"/>
+      <c r="K35" s="14">
+        <f>IF($A35="","",SUMPRODUCT(SUMIF(ShiftCode,D35:J35,ShiftHours)))</f>
+        <v/>
+      </c>
+      <c r="L35" s="25">
+        <f>IF($A35="","",IF(K35&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M35" s="14">
+        <f>IF($A35="","",MAX(R35:X35))</f>
+        <v/>
+      </c>
+      <c r="N35" s="25">
+        <f>IF($A35="","",IF(M35&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O35" s="14">
+        <f>IF($A35="","",IF(MIN(Z35:AE35)=999,"",MIN(Z35:AE35)))</f>
+        <v/>
+      </c>
+      <c r="P35" s="25">
+        <f>IF($A35="","",IF(AND(O35&lt;&gt;"",O35&lt;Rest_Hours),"SHORT",""))</f>
+        <v/>
+      </c>
+      <c r="Q35" s="25">
+        <f>IF($A35="","",IF(SUM(AG35:AM35)&gt;0,"CHECK",""))</f>
+        <v/>
+      </c>
+      <c r="R35">
+        <f>IF(SUMIF(ShiftCode,D35,ShiftHours)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="S35">
+        <f>IF(SUMIF(ShiftCode,E35,ShiftHours)&gt;0,R35+1,0)</f>
+        <v/>
+      </c>
+      <c r="T35">
+        <f>IF(SUMIF(ShiftCode,F35,ShiftHours)&gt;0,S35+1,0)</f>
+        <v/>
+      </c>
+      <c r="U35">
+        <f>IF(SUMIF(ShiftCode,G35,ShiftHours)&gt;0,T35+1,0)</f>
+        <v/>
+      </c>
+      <c r="V35">
+        <f>IF(SUMIF(ShiftCode,H35,ShiftHours)&gt;0,U35+1,0)</f>
+        <v/>
+      </c>
+      <c r="W35">
+        <f>IF(SUMIF(ShiftCode,I35,ShiftHours)&gt;0,V35+1,0)</f>
+        <v/>
+      </c>
+      <c r="X35">
+        <f>IF(SUMIF(ShiftCode,J35,ShiftHours)&gt;0,W35+1,0)</f>
+        <v/>
+      </c>
+      <c r="Z35">
+        <f>IF(AND(SUMIF(ShiftCode,D35,ShiftHours)&gt;0,SUMIF(ShiftCode,E35,ShiftHours)&gt;0),24+VLOOKUP(E35,ShiftFull,5,FALSE)-VLOOKUP(D35,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AA35">
+        <f>IF(AND(SUMIF(ShiftCode,E35,ShiftHours)&gt;0,SUMIF(ShiftCode,F35,ShiftHours)&gt;0),24+VLOOKUP(F35,ShiftFull,5,FALSE)-VLOOKUP(E35,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AB35">
+        <f>IF(AND(SUMIF(ShiftCode,F35,ShiftHours)&gt;0,SUMIF(ShiftCode,G35,ShiftHours)&gt;0),24+VLOOKUP(G35,ShiftFull,5,FALSE)-VLOOKUP(F35,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AC35">
+        <f>IF(AND(SUMIF(ShiftCode,G35,ShiftHours)&gt;0,SUMIF(ShiftCode,H35,ShiftHours)&gt;0),24+VLOOKUP(H35,ShiftFull,5,FALSE)-VLOOKUP(G35,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AD35">
+        <f>IF(AND(SUMIF(ShiftCode,H35,ShiftHours)&gt;0,SUMIF(ShiftCode,I35,ShiftHours)&gt;0),24+VLOOKUP(I35,ShiftFull,5,FALSE)-VLOOKUP(H35,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AE35">
+        <f>IF(AND(SUMIF(ShiftCode,I35,ShiftHours)&gt;0,SUMIF(ShiftCode,J35,ShiftHours)&gt;0),24+VLOOKUP(J35,ShiftFull,5,FALSE)-VLOOKUP(I35,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AG35">
+        <f>IF(AND(SUMIF(ShiftCode,D35,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A35)*(Leave!$B$2:$B$20&lt;=D$4)*(Leave!$C$2:$C$20&gt;=D$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AH35">
+        <f>IF(AND(SUMIF(ShiftCode,E35,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A35)*(Leave!$B$2:$B$20&lt;=E$4)*(Leave!$C$2:$C$20&gt;=E$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AI35">
+        <f>IF(AND(SUMIF(ShiftCode,F35,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A35)*(Leave!$B$2:$B$20&lt;=F$4)*(Leave!$C$2:$C$20&gt;=F$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AJ35">
+        <f>IF(AND(SUMIF(ShiftCode,G35,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A35)*(Leave!$B$2:$B$20&lt;=G$4)*(Leave!$C$2:$C$20&gt;=G$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AK35">
+        <f>IF(AND(SUMIF(ShiftCode,H35,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A35)*(Leave!$B$2:$B$20&lt;=H$4)*(Leave!$C$2:$C$20&gt;=H$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AL35">
+        <f>IF(AND(SUMIF(ShiftCode,I35,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A35)*(Leave!$B$2:$B$20&lt;=I$4)*(Leave!$C$2:$C$20&gt;=I$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AM35">
+        <f>IF(AND(SUMIF(ShiftCode,J35,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A35)*(Leave!$B$2:$B$20&lt;=J$4)*(Leave!$C$2:$C$20&gt;=J$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="15">
+        <f>IF(Staff!A26="","",Staff!A26)</f>
+        <v/>
+      </c>
+      <c r="B36" s="14">
+        <f>IF(A36="","",VLOOKUP(A36,StaffTbl,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D36" s="9" t="n"/>
+      <c r="E36" s="9" t="n"/>
+      <c r="F36" s="9" t="n"/>
+      <c r="G36" s="9" t="n"/>
+      <c r="H36" s="9" t="n"/>
+      <c r="I36" s="9" t="n"/>
+      <c r="J36" s="9" t="n"/>
+      <c r="K36" s="14">
+        <f>IF($A36="","",SUMPRODUCT(SUMIF(ShiftCode,D36:J36,ShiftHours)))</f>
+        <v/>
+      </c>
+      <c r="L36" s="25">
+        <f>IF($A36="","",IF(K36&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M36" s="14">
+        <f>IF($A36="","",MAX(R36:X36))</f>
+        <v/>
+      </c>
+      <c r="N36" s="25">
+        <f>IF($A36="","",IF(M36&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O36" s="14">
+        <f>IF($A36="","",IF(MIN(Z36:AE36)=999,"",MIN(Z36:AE36)))</f>
+        <v/>
+      </c>
+      <c r="P36" s="25">
+        <f>IF($A36="","",IF(AND(O36&lt;&gt;"",O36&lt;Rest_Hours),"SHORT",""))</f>
+        <v/>
+      </c>
+      <c r="Q36" s="25">
+        <f>IF($A36="","",IF(SUM(AG36:AM36)&gt;0,"CHECK",""))</f>
+        <v/>
+      </c>
+      <c r="R36">
+        <f>IF(SUMIF(ShiftCode,D36,ShiftHours)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="S36">
+        <f>IF(SUMIF(ShiftCode,E36,ShiftHours)&gt;0,R36+1,0)</f>
+        <v/>
+      </c>
+      <c r="T36">
+        <f>IF(SUMIF(ShiftCode,F36,ShiftHours)&gt;0,S36+1,0)</f>
+        <v/>
+      </c>
+      <c r="U36">
+        <f>IF(SUMIF(ShiftCode,G36,ShiftHours)&gt;0,T36+1,0)</f>
+        <v/>
+      </c>
+      <c r="V36">
+        <f>IF(SUMIF(ShiftCode,H36,ShiftHours)&gt;0,U36+1,0)</f>
+        <v/>
+      </c>
+      <c r="W36">
+        <f>IF(SUMIF(ShiftCode,I36,ShiftHours)&gt;0,V36+1,0)</f>
+        <v/>
+      </c>
+      <c r="X36">
+        <f>IF(SUMIF(ShiftCode,J36,ShiftHours)&gt;0,W36+1,0)</f>
+        <v/>
+      </c>
+      <c r="Z36">
+        <f>IF(AND(SUMIF(ShiftCode,D36,ShiftHours)&gt;0,SUMIF(ShiftCode,E36,ShiftHours)&gt;0),24+VLOOKUP(E36,ShiftFull,5,FALSE)-VLOOKUP(D36,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AA36">
+        <f>IF(AND(SUMIF(ShiftCode,E36,ShiftHours)&gt;0,SUMIF(ShiftCode,F36,ShiftHours)&gt;0),24+VLOOKUP(F36,ShiftFull,5,FALSE)-VLOOKUP(E36,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AB36">
+        <f>IF(AND(SUMIF(ShiftCode,F36,ShiftHours)&gt;0,SUMIF(ShiftCode,G36,ShiftHours)&gt;0),24+VLOOKUP(G36,ShiftFull,5,FALSE)-VLOOKUP(F36,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AC36">
+        <f>IF(AND(SUMIF(ShiftCode,G36,ShiftHours)&gt;0,SUMIF(ShiftCode,H36,ShiftHours)&gt;0),24+VLOOKUP(H36,ShiftFull,5,FALSE)-VLOOKUP(G36,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AD36">
+        <f>IF(AND(SUMIF(ShiftCode,H36,ShiftHours)&gt;0,SUMIF(ShiftCode,I36,ShiftHours)&gt;0),24+VLOOKUP(I36,ShiftFull,5,FALSE)-VLOOKUP(H36,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AE36">
+        <f>IF(AND(SUMIF(ShiftCode,I36,ShiftHours)&gt;0,SUMIF(ShiftCode,J36,ShiftHours)&gt;0),24+VLOOKUP(J36,ShiftFull,5,FALSE)-VLOOKUP(I36,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AG36">
+        <f>IF(AND(SUMIF(ShiftCode,D36,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A36)*(Leave!$B$2:$B$20&lt;=D$4)*(Leave!$C$2:$C$20&gt;=D$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AH36">
+        <f>IF(AND(SUMIF(ShiftCode,E36,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A36)*(Leave!$B$2:$B$20&lt;=E$4)*(Leave!$C$2:$C$20&gt;=E$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AI36">
+        <f>IF(AND(SUMIF(ShiftCode,F36,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A36)*(Leave!$B$2:$B$20&lt;=F$4)*(Leave!$C$2:$C$20&gt;=F$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AJ36">
+        <f>IF(AND(SUMIF(ShiftCode,G36,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A36)*(Leave!$B$2:$B$20&lt;=G$4)*(Leave!$C$2:$C$20&gt;=G$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AK36">
+        <f>IF(AND(SUMIF(ShiftCode,H36,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A36)*(Leave!$B$2:$B$20&lt;=H$4)*(Leave!$C$2:$C$20&gt;=H$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AL36">
+        <f>IF(AND(SUMIF(ShiftCode,I36,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A36)*(Leave!$B$2:$B$20&lt;=I$4)*(Leave!$C$2:$C$20&gt;=I$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AM36">
+        <f>IF(AND(SUMIF(ShiftCode,J36,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A36)*(Leave!$B$2:$B$20&lt;=J$4)*(Leave!$C$2:$C$20&gt;=J$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="15">
+        <f>IF(Staff!A27="","",Staff!A27)</f>
+        <v/>
+      </c>
+      <c r="B37" s="14">
+        <f>IF(A37="","",VLOOKUP(A37,StaffTbl,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D37" s="9" t="n"/>
+      <c r="E37" s="9" t="n"/>
+      <c r="F37" s="9" t="n"/>
+      <c r="G37" s="9" t="n"/>
+      <c r="H37" s="9" t="n"/>
+      <c r="I37" s="9" t="n"/>
+      <c r="J37" s="9" t="n"/>
+      <c r="K37" s="14">
+        <f>IF($A37="","",SUMPRODUCT(SUMIF(ShiftCode,D37:J37,ShiftHours)))</f>
+        <v/>
+      </c>
+      <c r="L37" s="25">
+        <f>IF($A37="","",IF(K37&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M37" s="14">
+        <f>IF($A37="","",MAX(R37:X37))</f>
+        <v/>
+      </c>
+      <c r="N37" s="25">
+        <f>IF($A37="","",IF(M37&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O37" s="14">
+        <f>IF($A37="","",IF(MIN(Z37:AE37)=999,"",MIN(Z37:AE37)))</f>
+        <v/>
+      </c>
+      <c r="P37" s="25">
+        <f>IF($A37="","",IF(AND(O37&lt;&gt;"",O37&lt;Rest_Hours),"SHORT",""))</f>
+        <v/>
+      </c>
+      <c r="Q37" s="25">
+        <f>IF($A37="","",IF(SUM(AG37:AM37)&gt;0,"CHECK",""))</f>
+        <v/>
+      </c>
+      <c r="R37">
+        <f>IF(SUMIF(ShiftCode,D37,ShiftHours)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="S37">
+        <f>IF(SUMIF(ShiftCode,E37,ShiftHours)&gt;0,R37+1,0)</f>
+        <v/>
+      </c>
+      <c r="T37">
+        <f>IF(SUMIF(ShiftCode,F37,ShiftHours)&gt;0,S37+1,0)</f>
+        <v/>
+      </c>
+      <c r="U37">
+        <f>IF(SUMIF(ShiftCode,G37,ShiftHours)&gt;0,T37+1,0)</f>
+        <v/>
+      </c>
+      <c r="V37">
+        <f>IF(SUMIF(ShiftCode,H37,ShiftHours)&gt;0,U37+1,0)</f>
+        <v/>
+      </c>
+      <c r="W37">
+        <f>IF(SUMIF(ShiftCode,I37,ShiftHours)&gt;0,V37+1,0)</f>
+        <v/>
+      </c>
+      <c r="X37">
+        <f>IF(SUMIF(ShiftCode,J37,ShiftHours)&gt;0,W37+1,0)</f>
+        <v/>
+      </c>
+      <c r="Z37">
+        <f>IF(AND(SUMIF(ShiftCode,D37,ShiftHours)&gt;0,SUMIF(ShiftCode,E37,ShiftHours)&gt;0),24+VLOOKUP(E37,ShiftFull,5,FALSE)-VLOOKUP(D37,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AA37">
+        <f>IF(AND(SUMIF(ShiftCode,E37,ShiftHours)&gt;0,SUMIF(ShiftCode,F37,ShiftHours)&gt;0),24+VLOOKUP(F37,ShiftFull,5,FALSE)-VLOOKUP(E37,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AB37">
+        <f>IF(AND(SUMIF(ShiftCode,F37,ShiftHours)&gt;0,SUMIF(ShiftCode,G37,ShiftHours)&gt;0),24+VLOOKUP(G37,ShiftFull,5,FALSE)-VLOOKUP(F37,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AC37">
+        <f>IF(AND(SUMIF(ShiftCode,G37,ShiftHours)&gt;0,SUMIF(ShiftCode,H37,ShiftHours)&gt;0),24+VLOOKUP(H37,ShiftFull,5,FALSE)-VLOOKUP(G37,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AD37">
+        <f>IF(AND(SUMIF(ShiftCode,H37,ShiftHours)&gt;0,SUMIF(ShiftCode,I37,ShiftHours)&gt;0),24+VLOOKUP(I37,ShiftFull,5,FALSE)-VLOOKUP(H37,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AE37">
+        <f>IF(AND(SUMIF(ShiftCode,I37,ShiftHours)&gt;0,SUMIF(ShiftCode,J37,ShiftHours)&gt;0),24+VLOOKUP(J37,ShiftFull,5,FALSE)-VLOOKUP(I37,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AG37">
+        <f>IF(AND(SUMIF(ShiftCode,D37,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A37)*(Leave!$B$2:$B$20&lt;=D$4)*(Leave!$C$2:$C$20&gt;=D$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AH37">
+        <f>IF(AND(SUMIF(ShiftCode,E37,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A37)*(Leave!$B$2:$B$20&lt;=E$4)*(Leave!$C$2:$C$20&gt;=E$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AI37">
+        <f>IF(AND(SUMIF(ShiftCode,F37,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A37)*(Leave!$B$2:$B$20&lt;=F$4)*(Leave!$C$2:$C$20&gt;=F$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AJ37">
+        <f>IF(AND(SUMIF(ShiftCode,G37,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A37)*(Leave!$B$2:$B$20&lt;=G$4)*(Leave!$C$2:$C$20&gt;=G$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AK37">
+        <f>IF(AND(SUMIF(ShiftCode,H37,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A37)*(Leave!$B$2:$B$20&lt;=H$4)*(Leave!$C$2:$C$20&gt;=H$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AL37">
+        <f>IF(AND(SUMIF(ShiftCode,I37,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A37)*(Leave!$B$2:$B$20&lt;=I$4)*(Leave!$C$2:$C$20&gt;=I$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AM37">
+        <f>IF(AND(SUMIF(ShiftCode,J37,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A37)*(Leave!$B$2:$B$20&lt;=J$4)*(Leave!$C$2:$C$20&gt;=J$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="15">
+        <f>IF(Staff!A28="","",Staff!A28)</f>
+        <v/>
+      </c>
+      <c r="B38" s="14">
+        <f>IF(A38="","",VLOOKUP(A38,StaffTbl,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D38" s="9" t="n"/>
+      <c r="E38" s="9" t="n"/>
+      <c r="F38" s="9" t="n"/>
+      <c r="G38" s="9" t="n"/>
+      <c r="H38" s="9" t="n"/>
+      <c r="I38" s="9" t="n"/>
+      <c r="J38" s="9" t="n"/>
+      <c r="K38" s="14">
+        <f>IF($A38="","",SUMPRODUCT(SUMIF(ShiftCode,D38:J38,ShiftHours)))</f>
+        <v/>
+      </c>
+      <c r="L38" s="25">
+        <f>IF($A38="","",IF(K38&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M38" s="14">
+        <f>IF($A38="","",MAX(R38:X38))</f>
+        <v/>
+      </c>
+      <c r="N38" s="25">
+        <f>IF($A38="","",IF(M38&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O38" s="14">
+        <f>IF($A38="","",IF(MIN(Z38:AE38)=999,"",MIN(Z38:AE38)))</f>
+        <v/>
+      </c>
+      <c r="P38" s="25">
+        <f>IF($A38="","",IF(AND(O38&lt;&gt;"",O38&lt;Rest_Hours),"SHORT",""))</f>
+        <v/>
+      </c>
+      <c r="Q38" s="25">
+        <f>IF($A38="","",IF(SUM(AG38:AM38)&gt;0,"CHECK",""))</f>
+        <v/>
+      </c>
+      <c r="R38">
+        <f>IF(SUMIF(ShiftCode,D38,ShiftHours)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="S38">
+        <f>IF(SUMIF(ShiftCode,E38,ShiftHours)&gt;0,R38+1,0)</f>
+        <v/>
+      </c>
+      <c r="T38">
+        <f>IF(SUMIF(ShiftCode,F38,ShiftHours)&gt;0,S38+1,0)</f>
+        <v/>
+      </c>
+      <c r="U38">
+        <f>IF(SUMIF(ShiftCode,G38,ShiftHours)&gt;0,T38+1,0)</f>
+        <v/>
+      </c>
+      <c r="V38">
+        <f>IF(SUMIF(ShiftCode,H38,ShiftHours)&gt;0,U38+1,0)</f>
+        <v/>
+      </c>
+      <c r="W38">
+        <f>IF(SUMIF(ShiftCode,I38,ShiftHours)&gt;0,V38+1,0)</f>
+        <v/>
+      </c>
+      <c r="X38">
+        <f>IF(SUMIF(ShiftCode,J38,ShiftHours)&gt;0,W38+1,0)</f>
+        <v/>
+      </c>
+      <c r="Z38">
+        <f>IF(AND(SUMIF(ShiftCode,D38,ShiftHours)&gt;0,SUMIF(ShiftCode,E38,ShiftHours)&gt;0),24+VLOOKUP(E38,ShiftFull,5,FALSE)-VLOOKUP(D38,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AA38">
+        <f>IF(AND(SUMIF(ShiftCode,E38,ShiftHours)&gt;0,SUMIF(ShiftCode,F38,ShiftHours)&gt;0),24+VLOOKUP(F38,ShiftFull,5,FALSE)-VLOOKUP(E38,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AB38">
+        <f>IF(AND(SUMIF(ShiftCode,F38,ShiftHours)&gt;0,SUMIF(ShiftCode,G38,ShiftHours)&gt;0),24+VLOOKUP(G38,ShiftFull,5,FALSE)-VLOOKUP(F38,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AC38">
+        <f>IF(AND(SUMIF(ShiftCode,G38,ShiftHours)&gt;0,SUMIF(ShiftCode,H38,ShiftHours)&gt;0),24+VLOOKUP(H38,ShiftFull,5,FALSE)-VLOOKUP(G38,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AD38">
+        <f>IF(AND(SUMIF(ShiftCode,H38,ShiftHours)&gt;0,SUMIF(ShiftCode,I38,ShiftHours)&gt;0),24+VLOOKUP(I38,ShiftFull,5,FALSE)-VLOOKUP(H38,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AE38">
+        <f>IF(AND(SUMIF(ShiftCode,I38,ShiftHours)&gt;0,SUMIF(ShiftCode,J38,ShiftHours)&gt;0),24+VLOOKUP(J38,ShiftFull,5,FALSE)-VLOOKUP(I38,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AG38">
+        <f>IF(AND(SUMIF(ShiftCode,D38,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A38)*(Leave!$B$2:$B$20&lt;=D$4)*(Leave!$C$2:$C$20&gt;=D$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AH38">
+        <f>IF(AND(SUMIF(ShiftCode,E38,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A38)*(Leave!$B$2:$B$20&lt;=E$4)*(Leave!$C$2:$C$20&gt;=E$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AI38">
+        <f>IF(AND(SUMIF(ShiftCode,F38,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A38)*(Leave!$B$2:$B$20&lt;=F$4)*(Leave!$C$2:$C$20&gt;=F$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AJ38">
+        <f>IF(AND(SUMIF(ShiftCode,G38,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A38)*(Leave!$B$2:$B$20&lt;=G$4)*(Leave!$C$2:$C$20&gt;=G$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AK38">
+        <f>IF(AND(SUMIF(ShiftCode,H38,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A38)*(Leave!$B$2:$B$20&lt;=H$4)*(Leave!$C$2:$C$20&gt;=H$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AL38">
+        <f>IF(AND(SUMIF(ShiftCode,I38,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A38)*(Leave!$B$2:$B$20&lt;=I$4)*(Leave!$C$2:$C$20&gt;=I$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AM38">
+        <f>IF(AND(SUMIF(ShiftCode,J38,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A38)*(Leave!$B$2:$B$20&lt;=J$4)*(Leave!$C$2:$C$20&gt;=J$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="15">
+        <f>IF(Staff!A29="","",Staff!A29)</f>
+        <v/>
+      </c>
+      <c r="B39" s="14">
+        <f>IF(A39="","",VLOOKUP(A39,StaffTbl,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D39" s="9" t="n"/>
+      <c r="E39" s="9" t="n"/>
+      <c r="F39" s="9" t="n"/>
+      <c r="G39" s="9" t="n"/>
+      <c r="H39" s="9" t="n"/>
+      <c r="I39" s="9" t="n"/>
+      <c r="J39" s="9" t="n"/>
+      <c r="K39" s="14">
+        <f>IF($A39="","",SUMPRODUCT(SUMIF(ShiftCode,D39:J39,ShiftHours)))</f>
+        <v/>
+      </c>
+      <c r="L39" s="25">
+        <f>IF($A39="","",IF(K39&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M39" s="14">
+        <f>IF($A39="","",MAX(R39:X39))</f>
+        <v/>
+      </c>
+      <c r="N39" s="25">
+        <f>IF($A39="","",IF(M39&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O39" s="14">
+        <f>IF($A39="","",IF(MIN(Z39:AE39)=999,"",MIN(Z39:AE39)))</f>
+        <v/>
+      </c>
+      <c r="P39" s="25">
+        <f>IF($A39="","",IF(AND(O39&lt;&gt;"",O39&lt;Rest_Hours),"SHORT",""))</f>
+        <v/>
+      </c>
+      <c r="Q39" s="25">
+        <f>IF($A39="","",IF(SUM(AG39:AM39)&gt;0,"CHECK",""))</f>
+        <v/>
+      </c>
+      <c r="R39">
+        <f>IF(SUMIF(ShiftCode,D39,ShiftHours)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="S39">
+        <f>IF(SUMIF(ShiftCode,E39,ShiftHours)&gt;0,R39+1,0)</f>
+        <v/>
+      </c>
+      <c r="T39">
+        <f>IF(SUMIF(ShiftCode,F39,ShiftHours)&gt;0,S39+1,0)</f>
+        <v/>
+      </c>
+      <c r="U39">
+        <f>IF(SUMIF(ShiftCode,G39,ShiftHours)&gt;0,T39+1,0)</f>
+        <v/>
+      </c>
+      <c r="V39">
+        <f>IF(SUMIF(ShiftCode,H39,ShiftHours)&gt;0,U39+1,0)</f>
+        <v/>
+      </c>
+      <c r="W39">
+        <f>IF(SUMIF(ShiftCode,I39,ShiftHours)&gt;0,V39+1,0)</f>
+        <v/>
+      </c>
+      <c r="X39">
+        <f>IF(SUMIF(ShiftCode,J39,ShiftHours)&gt;0,W39+1,0)</f>
+        <v/>
+      </c>
+      <c r="Z39">
+        <f>IF(AND(SUMIF(ShiftCode,D39,ShiftHours)&gt;0,SUMIF(ShiftCode,E39,ShiftHours)&gt;0),24+VLOOKUP(E39,ShiftFull,5,FALSE)-VLOOKUP(D39,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AA39">
+        <f>IF(AND(SUMIF(ShiftCode,E39,ShiftHours)&gt;0,SUMIF(ShiftCode,F39,ShiftHours)&gt;0),24+VLOOKUP(F39,ShiftFull,5,FALSE)-VLOOKUP(E39,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AB39">
+        <f>IF(AND(SUMIF(ShiftCode,F39,ShiftHours)&gt;0,SUMIF(ShiftCode,G39,ShiftHours)&gt;0),24+VLOOKUP(G39,ShiftFull,5,FALSE)-VLOOKUP(F39,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AC39">
+        <f>IF(AND(SUMIF(ShiftCode,G39,ShiftHours)&gt;0,SUMIF(ShiftCode,H39,ShiftHours)&gt;0),24+VLOOKUP(H39,ShiftFull,5,FALSE)-VLOOKUP(G39,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AD39">
+        <f>IF(AND(SUMIF(ShiftCode,H39,ShiftHours)&gt;0,SUMIF(ShiftCode,I39,ShiftHours)&gt;0),24+VLOOKUP(I39,ShiftFull,5,FALSE)-VLOOKUP(H39,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AE39">
+        <f>IF(AND(SUMIF(ShiftCode,I39,ShiftHours)&gt;0,SUMIF(ShiftCode,J39,ShiftHours)&gt;0),24+VLOOKUP(J39,ShiftFull,5,FALSE)-VLOOKUP(I39,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AG39">
+        <f>IF(AND(SUMIF(ShiftCode,D39,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A39)*(Leave!$B$2:$B$20&lt;=D$4)*(Leave!$C$2:$C$20&gt;=D$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AH39">
+        <f>IF(AND(SUMIF(ShiftCode,E39,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A39)*(Leave!$B$2:$B$20&lt;=E$4)*(Leave!$C$2:$C$20&gt;=E$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AI39">
+        <f>IF(AND(SUMIF(ShiftCode,F39,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A39)*(Leave!$B$2:$B$20&lt;=F$4)*(Leave!$C$2:$C$20&gt;=F$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AJ39">
+        <f>IF(AND(SUMIF(ShiftCode,G39,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A39)*(Leave!$B$2:$B$20&lt;=G$4)*(Leave!$C$2:$C$20&gt;=G$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AK39">
+        <f>IF(AND(SUMIF(ShiftCode,H39,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A39)*(Leave!$B$2:$B$20&lt;=H$4)*(Leave!$C$2:$C$20&gt;=H$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AL39">
+        <f>IF(AND(SUMIF(ShiftCode,I39,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A39)*(Leave!$B$2:$B$20&lt;=I$4)*(Leave!$C$2:$C$20&gt;=I$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AM39">
+        <f>IF(AND(SUMIF(ShiftCode,J39,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A39)*(Leave!$B$2:$B$20&lt;=J$4)*(Leave!$C$2:$C$20&gt;=J$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="15">
+        <f>IF(Staff!A30="","",Staff!A30)</f>
+        <v/>
+      </c>
+      <c r="B40" s="14">
+        <f>IF(A40="","",VLOOKUP(A40,StaffTbl,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D40" s="9" t="n"/>
+      <c r="E40" s="9" t="n"/>
+      <c r="F40" s="9" t="n"/>
+      <c r="G40" s="9" t="n"/>
+      <c r="H40" s="9" t="n"/>
+      <c r="I40" s="9" t="n"/>
+      <c r="J40" s="9" t="n"/>
+      <c r="K40" s="14">
+        <f>IF($A40="","",SUMPRODUCT(SUMIF(ShiftCode,D40:J40,ShiftHours)))</f>
+        <v/>
+      </c>
+      <c r="L40" s="25">
+        <f>IF($A40="","",IF(K40&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M40" s="14">
+        <f>IF($A40="","",MAX(R40:X40))</f>
+        <v/>
+      </c>
+      <c r="N40" s="25">
+        <f>IF($A40="","",IF(M40&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O40" s="14">
+        <f>IF($A40="","",IF(MIN(Z40:AE40)=999,"",MIN(Z40:AE40)))</f>
+        <v/>
+      </c>
+      <c r="P40" s="25">
+        <f>IF($A40="","",IF(AND(O40&lt;&gt;"",O40&lt;Rest_Hours),"SHORT",""))</f>
+        <v/>
+      </c>
+      <c r="Q40" s="25">
+        <f>IF($A40="","",IF(SUM(AG40:AM40)&gt;0,"CHECK",""))</f>
+        <v/>
+      </c>
+      <c r="R40">
+        <f>IF(SUMIF(ShiftCode,D40,ShiftHours)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="S40">
+        <f>IF(SUMIF(ShiftCode,E40,ShiftHours)&gt;0,R40+1,0)</f>
+        <v/>
+      </c>
+      <c r="T40">
+        <f>IF(SUMIF(ShiftCode,F40,ShiftHours)&gt;0,S40+1,0)</f>
+        <v/>
+      </c>
+      <c r="U40">
+        <f>IF(SUMIF(ShiftCode,G40,ShiftHours)&gt;0,T40+1,0)</f>
+        <v/>
+      </c>
+      <c r="V40">
+        <f>IF(SUMIF(ShiftCode,H40,ShiftHours)&gt;0,U40+1,0)</f>
+        <v/>
+      </c>
+      <c r="W40">
+        <f>IF(SUMIF(ShiftCode,I40,ShiftHours)&gt;0,V40+1,0)</f>
+        <v/>
+      </c>
+      <c r="X40">
+        <f>IF(SUMIF(ShiftCode,J40,ShiftHours)&gt;0,W40+1,0)</f>
+        <v/>
+      </c>
+      <c r="Z40">
+        <f>IF(AND(SUMIF(ShiftCode,D40,ShiftHours)&gt;0,SUMIF(ShiftCode,E40,ShiftHours)&gt;0),24+VLOOKUP(E40,ShiftFull,5,FALSE)-VLOOKUP(D40,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AA40">
+        <f>IF(AND(SUMIF(ShiftCode,E40,ShiftHours)&gt;0,SUMIF(ShiftCode,F40,ShiftHours)&gt;0),24+VLOOKUP(F40,ShiftFull,5,FALSE)-VLOOKUP(E40,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AB40">
+        <f>IF(AND(SUMIF(ShiftCode,F40,ShiftHours)&gt;0,SUMIF(ShiftCode,G40,ShiftHours)&gt;0),24+VLOOKUP(G40,ShiftFull,5,FALSE)-VLOOKUP(F40,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AC40">
+        <f>IF(AND(SUMIF(ShiftCode,G40,ShiftHours)&gt;0,SUMIF(ShiftCode,H40,ShiftHours)&gt;0),24+VLOOKUP(H40,ShiftFull,5,FALSE)-VLOOKUP(G40,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AD40">
+        <f>IF(AND(SUMIF(ShiftCode,H40,ShiftHours)&gt;0,SUMIF(ShiftCode,I40,ShiftHours)&gt;0),24+VLOOKUP(I40,ShiftFull,5,FALSE)-VLOOKUP(H40,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AE40">
+        <f>IF(AND(SUMIF(ShiftCode,I40,ShiftHours)&gt;0,SUMIF(ShiftCode,J40,ShiftHours)&gt;0),24+VLOOKUP(J40,ShiftFull,5,FALSE)-VLOOKUP(I40,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AG40">
+        <f>IF(AND(SUMIF(ShiftCode,D40,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A40)*(Leave!$B$2:$B$20&lt;=D$4)*(Leave!$C$2:$C$20&gt;=D$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AH40">
+        <f>IF(AND(SUMIF(ShiftCode,E40,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A40)*(Leave!$B$2:$B$20&lt;=E$4)*(Leave!$C$2:$C$20&gt;=E$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AI40">
+        <f>IF(AND(SUMIF(ShiftCode,F40,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A40)*(Leave!$B$2:$B$20&lt;=F$4)*(Leave!$C$2:$C$20&gt;=F$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AJ40">
+        <f>IF(AND(SUMIF(ShiftCode,G40,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A40)*(Leave!$B$2:$B$20&lt;=G$4)*(Leave!$C$2:$C$20&gt;=G$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AK40">
+        <f>IF(AND(SUMIF(ShiftCode,H40,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A40)*(Leave!$B$2:$B$20&lt;=H$4)*(Leave!$C$2:$C$20&gt;=H$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AL40">
+        <f>IF(AND(SUMIF(ShiftCode,I40,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A40)*(Leave!$B$2:$B$20&lt;=I$4)*(Leave!$C$2:$C$20&gt;=I$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AM40">
+        <f>IF(AND(SUMIF(ShiftCode,J40,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A40)*(Leave!$B$2:$B$20&lt;=J$4)*(Leave!$C$2:$C$20&gt;=J$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="15">
+        <f>IF(Staff!A31="","",Staff!A31)</f>
+        <v/>
+      </c>
+      <c r="B41" s="14">
+        <f>IF(A41="","",VLOOKUP(A41,StaffTbl,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D41" s="9" t="n"/>
+      <c r="E41" s="9" t="n"/>
+      <c r="F41" s="9" t="n"/>
+      <c r="G41" s="9" t="n"/>
+      <c r="H41" s="9" t="n"/>
+      <c r="I41" s="9" t="n"/>
+      <c r="J41" s="9" t="n"/>
+      <c r="K41" s="14">
+        <f>IF($A41="","",SUMPRODUCT(SUMIF(ShiftCode,D41:J41,ShiftHours)))</f>
+        <v/>
+      </c>
+      <c r="L41" s="25">
+        <f>IF($A41="","",IF(K41&gt;OT_Threshold,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="M41" s="14">
+        <f>IF($A41="","",MAX(R41:X41))</f>
+        <v/>
+      </c>
+      <c r="N41" s="25">
+        <f>IF($A41="","",IF(M41&gt;Max_Consecutive,"OVER",""))</f>
+        <v/>
+      </c>
+      <c r="O41" s="14">
+        <f>IF($A41="","",IF(MIN(Z41:AE41)=999,"",MIN(Z41:AE41)))</f>
+        <v/>
+      </c>
+      <c r="P41" s="25">
+        <f>IF($A41="","",IF(AND(O41&lt;&gt;"",O41&lt;Rest_Hours),"SHORT",""))</f>
+        <v/>
+      </c>
+      <c r="Q41" s="25">
+        <f>IF($A41="","",IF(SUM(AG41:AM41)&gt;0,"CHECK",""))</f>
+        <v/>
+      </c>
+      <c r="R41">
+        <f>IF(SUMIF(ShiftCode,D41,ShiftHours)&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="S41">
+        <f>IF(SUMIF(ShiftCode,E41,ShiftHours)&gt;0,R41+1,0)</f>
+        <v/>
+      </c>
+      <c r="T41">
+        <f>IF(SUMIF(ShiftCode,F41,ShiftHours)&gt;0,S41+1,0)</f>
+        <v/>
+      </c>
+      <c r="U41">
+        <f>IF(SUMIF(ShiftCode,G41,ShiftHours)&gt;0,T41+1,0)</f>
+        <v/>
+      </c>
+      <c r="V41">
+        <f>IF(SUMIF(ShiftCode,H41,ShiftHours)&gt;0,U41+1,0)</f>
+        <v/>
+      </c>
+      <c r="W41">
+        <f>IF(SUMIF(ShiftCode,I41,ShiftHours)&gt;0,V41+1,0)</f>
+        <v/>
+      </c>
+      <c r="X41">
+        <f>IF(SUMIF(ShiftCode,J41,ShiftHours)&gt;0,W41+1,0)</f>
+        <v/>
+      </c>
+      <c r="Z41">
+        <f>IF(AND(SUMIF(ShiftCode,D41,ShiftHours)&gt;0,SUMIF(ShiftCode,E41,ShiftHours)&gt;0),24+VLOOKUP(E41,ShiftFull,5,FALSE)-VLOOKUP(D41,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AA41">
+        <f>IF(AND(SUMIF(ShiftCode,E41,ShiftHours)&gt;0,SUMIF(ShiftCode,F41,ShiftHours)&gt;0),24+VLOOKUP(F41,ShiftFull,5,FALSE)-VLOOKUP(E41,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AB41">
+        <f>IF(AND(SUMIF(ShiftCode,F41,ShiftHours)&gt;0,SUMIF(ShiftCode,G41,ShiftHours)&gt;0),24+VLOOKUP(G41,ShiftFull,5,FALSE)-VLOOKUP(F41,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AC41">
+        <f>IF(AND(SUMIF(ShiftCode,G41,ShiftHours)&gt;0,SUMIF(ShiftCode,H41,ShiftHours)&gt;0),24+VLOOKUP(H41,ShiftFull,5,FALSE)-VLOOKUP(G41,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AD41">
+        <f>IF(AND(SUMIF(ShiftCode,H41,ShiftHours)&gt;0,SUMIF(ShiftCode,I41,ShiftHours)&gt;0),24+VLOOKUP(I41,ShiftFull,5,FALSE)-VLOOKUP(H41,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AE41">
+        <f>IF(AND(SUMIF(ShiftCode,I41,ShiftHours)&gt;0,SUMIF(ShiftCode,J41,ShiftHours)&gt;0),24+VLOOKUP(J41,ShiftFull,5,FALSE)-VLOOKUP(I41,ShiftFull,6,FALSE),999)</f>
+        <v/>
+      </c>
+      <c r="AG41">
+        <f>IF(AND(SUMIF(ShiftCode,D41,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A41)*(Leave!$B$2:$B$20&lt;=D$4)*(Leave!$C$2:$C$20&gt;=D$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AH41">
+        <f>IF(AND(SUMIF(ShiftCode,E41,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A41)*(Leave!$B$2:$B$20&lt;=E$4)*(Leave!$C$2:$C$20&gt;=E$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AI41">
+        <f>IF(AND(SUMIF(ShiftCode,F41,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A41)*(Leave!$B$2:$B$20&lt;=F$4)*(Leave!$C$2:$C$20&gt;=F$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AJ41">
+        <f>IF(AND(SUMIF(ShiftCode,G41,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A41)*(Leave!$B$2:$B$20&lt;=G$4)*(Leave!$C$2:$C$20&gt;=G$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AK41">
+        <f>IF(AND(SUMIF(ShiftCode,H41,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A41)*(Leave!$B$2:$B$20&lt;=H$4)*(Leave!$C$2:$C$20&gt;=H$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AL41">
+        <f>IF(AND(SUMIF(ShiftCode,I41,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A41)*(Leave!$B$2:$B$20&lt;=I$4)*(Leave!$C$2:$C$20&gt;=I$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+      <c r="AM41">
+        <f>IF(AND(SUMIF(ShiftCode,J41,ShiftHours)&gt;0,SUMPRODUCT((Leave!$A$2:$A$20=$A41)*(Leave!$B$2:$B$20&lt;=J$4)*(Leave!$C$2:$C$20&gt;=J$4))&gt;0),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="20" t="inlineStr">
         <is>
           <t>Assigned RN - Day</t>
         </is>
       </c>
-      <c r="D33" s="13">
-        <f>SUMPRODUCT(($B$12:$B$31="RN")*(COUNTIF(DayCodes,D12:D31)&gt;0))</f>
-        <v/>
-      </c>
-      <c r="E33" s="13">
-        <f>SUMPRODUCT(($B$12:$B$31="RN")*(COUNTIF(DayCodes,E12:E31)&gt;0))</f>
-        <v/>
-      </c>
-      <c r="F33" s="13">
-        <f>SUMPRODUCT(($B$12:$B$31="RN")*(COUNTIF(DayCodes,F12:F31)&gt;0))</f>
-        <v/>
-      </c>
-      <c r="G33" s="13">
-        <f>SUMPRODUCT(($B$12:$B$31="RN")*(COUNTIF(DayCodes,G12:G31)&gt;0))</f>
-        <v/>
-      </c>
-      <c r="H33" s="13">
-        <f>SUMPRODUCT(($B$12:$B$31="RN")*(COUNTIF(DayCodes,H12:H31)&gt;0))</f>
-        <v/>
-      </c>
-      <c r="I33" s="13">
-        <f>SUMPRODUCT(($B$12:$B$31="RN")*(COUNTIF(DayCodes,I12:I31)&gt;0))</f>
-        <v/>
-      </c>
-      <c r="J33" s="13">
-        <f>SUMPRODUCT(($B$12:$B$31="RN")*(COUNTIF(DayCodes,J12:J31)&gt;0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="20" t="inlineStr">
+      <c r="D43" s="14">
+        <f>SUMPRODUCT(($B$12:$B$41="RN")*(COUNTIF(DayCodes,D12:D41)&gt;0))</f>
+        <v/>
+      </c>
+      <c r="E43" s="14">
+        <f>SUMPRODUCT(($B$12:$B$41="RN")*(COUNTIF(DayCodes,E12:E41)&gt;0))</f>
+        <v/>
+      </c>
+      <c r="F43" s="14">
+        <f>SUMPRODUCT(($B$12:$B$41="RN")*(COUNTIF(DayCodes,F12:F41)&gt;0))</f>
+        <v/>
+      </c>
+      <c r="G43" s="14">
+        <f>SUMPRODUCT(($B$12:$B$41="RN")*(COUNTIF(DayCodes,G12:G41)&gt;0))</f>
+        <v/>
+      </c>
+      <c r="H43" s="14">
+        <f>SUMPRODUCT(($B$12:$B$41="RN")*(COUNTIF(DayCodes,H12:H41)&gt;0))</f>
+        <v/>
+      </c>
+      <c r="I43" s="14">
+        <f>SUMPRODUCT(($B$12:$B$41="RN")*(COUNTIF(DayCodes,I12:I41)&gt;0))</f>
+        <v/>
+      </c>
+      <c r="J43" s="14">
+        <f>SUMPRODUCT(($B$12:$B$41="RN")*(COUNTIF(DayCodes,J12:J41)&gt;0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="20" t="inlineStr">
         <is>
           <t>Assigned RN - Night</t>
         </is>
       </c>
-      <c r="D34" s="13">
-        <f>SUMPRODUCT(($B$12:$B$31="RN")*(COUNTIF(NightCodes,D12:D31)&gt;0))</f>
-        <v/>
-      </c>
-      <c r="E34" s="13">
-        <f>SUMPRODUCT(($B$12:$B$31="RN")*(COUNTIF(NightCodes,E12:E31)&gt;0))</f>
-        <v/>
-      </c>
-      <c r="F34" s="13">
-        <f>SUMPRODUCT(($B$12:$B$31="RN")*(COUNTIF(NightCodes,F12:F31)&gt;0))</f>
-        <v/>
-      </c>
-      <c r="G34" s="13">
-        <f>SUMPRODUCT(($B$12:$B$31="RN")*(COUNTIF(NightCodes,G12:G31)&gt;0))</f>
-        <v/>
-      </c>
-      <c r="H34" s="13">
-        <f>SUMPRODUCT(($B$12:$B$31="RN")*(COUNTIF(NightCodes,H12:H31)&gt;0))</f>
-        <v/>
-      </c>
-      <c r="I34" s="13">
-        <f>SUMPRODUCT(($B$12:$B$31="RN")*(COUNTIF(NightCodes,I12:I31)&gt;0))</f>
-        <v/>
-      </c>
-      <c r="J34" s="13">
-        <f>SUMPRODUCT(($B$12:$B$31="RN")*(COUNTIF(NightCodes,J12:J31)&gt;0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="26" t="inlineStr">
+      <c r="D44" s="14">
+        <f>SUMPRODUCT(($B$12:$B$41="RN")*(COUNTIF(NightCodes,D12:D41)&gt;0))</f>
+        <v/>
+      </c>
+      <c r="E44" s="14">
+        <f>SUMPRODUCT(($B$12:$B$41="RN")*(COUNTIF(NightCodes,E12:E41)&gt;0))</f>
+        <v/>
+      </c>
+      <c r="F44" s="14">
+        <f>SUMPRODUCT(($B$12:$B$41="RN")*(COUNTIF(NightCodes,F12:F41)&gt;0))</f>
+        <v/>
+      </c>
+      <c r="G44" s="14">
+        <f>SUMPRODUCT(($B$12:$B$41="RN")*(COUNTIF(NightCodes,G12:G41)&gt;0))</f>
+        <v/>
+      </c>
+      <c r="H44" s="14">
+        <f>SUMPRODUCT(($B$12:$B$41="RN")*(COUNTIF(NightCodes,H12:H41)&gt;0))</f>
+        <v/>
+      </c>
+      <c r="I44" s="14">
+        <f>SUMPRODUCT(($B$12:$B$41="RN")*(COUNTIF(NightCodes,I12:I41)&gt;0))</f>
+        <v/>
+      </c>
+      <c r="J44" s="14">
+        <f>SUMPRODUCT(($B$12:$B$41="RN")*(COUNTIF(NightCodes,J12:J41)&gt;0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="26" t="inlineStr">
         <is>
           <t>Coverage gap - Day (RN, + = short)</t>
         </is>
       </c>
-      <c r="D35" s="13">
-        <f>D6-D33</f>
-        <v/>
-      </c>
-      <c r="E35" s="13">
-        <f>E6-E33</f>
-        <v/>
-      </c>
-      <c r="F35" s="13">
-        <f>F6-F33</f>
-        <v/>
-      </c>
-      <c r="G35" s="13">
-        <f>G6-G33</f>
-        <v/>
-      </c>
-      <c r="H35" s="13">
-        <f>H6-H33</f>
-        <v/>
-      </c>
-      <c r="I35" s="13">
-        <f>I6-I33</f>
-        <v/>
-      </c>
-      <c r="J35" s="13">
-        <f>J6-J33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="26" t="inlineStr">
+      <c r="D45" s="14">
+        <f>D6-D43</f>
+        <v/>
+      </c>
+      <c r="E45" s="14">
+        <f>E6-E43</f>
+        <v/>
+      </c>
+      <c r="F45" s="14">
+        <f>F6-F43</f>
+        <v/>
+      </c>
+      <c r="G45" s="14">
+        <f>G6-G43</f>
+        <v/>
+      </c>
+      <c r="H45" s="14">
+        <f>H6-H43</f>
+        <v/>
+      </c>
+      <c r="I45" s="14">
+        <f>I6-I43</f>
+        <v/>
+      </c>
+      <c r="J45" s="14">
+        <f>J6-J43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="26" t="inlineStr">
         <is>
           <t>Coverage gap - Night (RN, + = short)</t>
         </is>
       </c>
-      <c r="D36" s="13">
-        <f>D7-D34</f>
-        <v/>
-      </c>
-      <c r="E36" s="13">
-        <f>E7-E34</f>
-        <v/>
-      </c>
-      <c r="F36" s="13">
-        <f>F7-F34</f>
-        <v/>
-      </c>
-      <c r="G36" s="13">
-        <f>G7-G34</f>
-        <v/>
-      </c>
-      <c r="H36" s="13">
-        <f>H7-H34</f>
-        <v/>
-      </c>
-      <c r="I36" s="13">
-        <f>I7-I34</f>
-        <v/>
-      </c>
-      <c r="J36" s="13">
-        <f>J7-J34</f>
+      <c r="D46" s="14">
+        <f>D7-D44</f>
+        <v/>
+      </c>
+      <c r="E46" s="14">
+        <f>E7-E44</f>
+        <v/>
+      </c>
+      <c r="F46" s="14">
+        <f>F7-F44</f>
+        <v/>
+      </c>
+      <c r="G46" s="14">
+        <f>G7-G44</f>
+        <v/>
+      </c>
+      <c r="H46" s="14">
+        <f>H7-H44</f>
+        <v/>
+      </c>
+      <c r="I46" s="14">
+        <f>I7-I44</f>
+        <v/>
+      </c>
+      <c r="J46" s="14">
+        <f>J7-J44</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1" password="8610"/>
-  <conditionalFormatting sqref="D12:J31">
+  <conditionalFormatting sqref="D12:J41">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>COUNTIF(DayCodes,D12)&gt;0</formula>
     </cfRule>
@@ -6338,32 +7712,32 @@
       <formula>COUNTIF(OffCodes,D12)&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L12:L31">
+  <conditionalFormatting sqref="L12:L41">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"OVER"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N12:N31">
+  <conditionalFormatting sqref="N12:N41">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="3">
       <formula>"OVER"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P12:P31">
+  <conditionalFormatting sqref="P12:P41">
     <cfRule type="cellIs" priority="6" operator="equal" dxfId="3">
       <formula>"SHORT"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q12:Q31">
+  <conditionalFormatting sqref="Q12:Q41">
     <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
       <formula>"CHECK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D35:J35">
+  <conditionalFormatting sqref="D45:J45">
     <cfRule type="cellIs" priority="8" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D36:J36">
+  <conditionalFormatting sqref="D46:J46">
     <cfRule type="cellIs" priority="9" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6374,7 +7748,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="D12:J31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D12:J41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>ShiftCode</formula1>
     </dataValidation>
     <dataValidation sqref="B1" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">

</xml_diff>